<commit_message>
Change make file to compile all C files together. Updated Readme file. Updated python and results. Regenerated esop results.
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maslov Cost" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T-Count" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,25 +426,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Benchmark</t>
+          <t>Function</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Inputs</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>ESOP Cost</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>ESOP T</t>
-        </is>
-      </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EOSOPS Cost</t>
@@ -451,27 +452,17 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>EOSOPS T</t>
+          <t>EOSOPS Cost Saving (%)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>EOSOPS Savings %</t>
+          <t>Final Cost</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>FINAL Cost</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>FINAL T</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>FINAL Savings %</t>
+          <t>Final Cost Saving (%)</t>
         </is>
       </c>
     </row>
@@ -482,28 +473,1173 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" t="n">
         <v>857</v>
+      </c>
+      <c r="D2" t="n">
+        <v>603</v>
+      </c>
+      <c r="E2" t="n">
+        <v>29.64</v>
+      </c>
+      <c r="F2" t="n">
+        <v>207</v>
+      </c>
+      <c r="G2" t="n">
+        <v>75.84999999999999</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>9sym_d_100</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C3" t="n">
+        <v>21212</v>
+      </c>
+      <c r="D3" t="n">
+        <v>12524</v>
+      </c>
+      <c r="E3" t="n">
+        <v>40.96</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3519</v>
+      </c>
+      <c r="G3" t="n">
+        <v>83.41</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>con1f1_100</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" t="n">
+        <v>141</v>
+      </c>
+      <c r="D4" t="n">
+        <v>114</v>
+      </c>
+      <c r="E4" t="n">
+        <v>19.15</v>
+      </c>
+      <c r="F4" t="n">
+        <v>43</v>
+      </c>
+      <c r="G4" t="n">
+        <v>69.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>con2f2_100</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C5" t="n">
+        <v>68</v>
+      </c>
+      <c r="D5" t="n">
+        <v>68</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>45</v>
+      </c>
+      <c r="G5" t="n">
+        <v>33.82</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>eosops1_100</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>68</v>
+      </c>
+      <c r="D6" t="n">
+        <v>22</v>
+      </c>
+      <c r="E6" t="n">
+        <v>67.65000000000001</v>
+      </c>
+      <c r="F6" t="n">
+        <v>22</v>
+      </c>
+      <c r="G6" t="n">
+        <v>67.65000000000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>exam1_d_100</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>exam3_d_100</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>39</v>
+      </c>
+      <c r="D8" t="n">
+        <v>39</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>24</v>
+      </c>
+      <c r="G8" t="n">
+        <v>38.46</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>life_d_100</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" t="n">
+        <v>13108</v>
+      </c>
+      <c r="D9" t="n">
+        <v>7680</v>
+      </c>
+      <c r="E9" t="n">
+        <v>41.41</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2464</v>
+      </c>
+      <c r="G9" t="n">
+        <v>81.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>max46_d_100</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="n">
+        <v>14378</v>
+      </c>
+      <c r="D10" t="n">
+        <v>12322</v>
+      </c>
+      <c r="E10" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2487</v>
+      </c>
+      <c r="G10" t="n">
+        <v>82.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>newill_d_100</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1239</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1239</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>230</v>
+      </c>
+      <c r="G11" t="n">
+        <v>81.44</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>newtag_d_100</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>683</v>
+      </c>
+      <c r="D12" t="n">
+        <v>683</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>161</v>
+      </c>
+      <c r="G12" t="n">
+        <v>76.43000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>rd53f1_100</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>185</v>
+      </c>
+      <c r="D13" t="n">
+        <v>75</v>
+      </c>
+      <c r="E13" t="n">
+        <v>59.46</v>
+      </c>
+      <c r="F13" t="n">
+        <v>75</v>
+      </c>
+      <c r="G13" t="n">
+        <v>59.46</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>rd53f2_100</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" t="n">
+        <v>88</v>
+      </c>
+      <c r="D14" t="n">
+        <v>88</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>47</v>
+      </c>
+      <c r="G14" t="n">
+        <v>46.59</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>rd53f3_100</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" t="n">
+        <v>13</v>
+      </c>
+      <c r="D15" t="n">
+        <v>13</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>13</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>rd73f1_100</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7</v>
+      </c>
+      <c r="C16" t="n">
+        <v>211</v>
+      </c>
+      <c r="D16" t="n">
+        <v>211</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>106</v>
+      </c>
+      <c r="G16" t="n">
+        <v>49.76</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>rd73f2_100</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>7</v>
+      </c>
+      <c r="C17" t="n">
+        <v>19</v>
+      </c>
+      <c r="D17" t="n">
+        <v>19</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>19</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>rd73f3_100</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1341</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1318</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="F18" t="n">
+        <v>339</v>
+      </c>
+      <c r="G18" t="n">
+        <v>74.72</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>rd84f1_100</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" t="n">
+        <v>277</v>
+      </c>
+      <c r="D19" t="n">
+        <v>277</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>127</v>
+      </c>
+      <c r="G19" t="n">
+        <v>54.15</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>rd84f2_100</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="n">
+        <v>24</v>
+      </c>
+      <c r="D20" t="n">
+        <v>24</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>24</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>rd84f3_100</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" t="n">
+        <v>509</v>
+      </c>
+      <c r="D21" t="n">
+        <v>509</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>509</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>rd84f4_100</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>8</v>
+      </c>
+      <c r="C22" t="n">
+        <v>4696</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2898</v>
+      </c>
+      <c r="E22" t="n">
+        <v>38.29</v>
+      </c>
+      <c r="F22" t="n">
+        <v>910</v>
+      </c>
+      <c r="G22" t="n">
+        <v>80.62</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>sao2f1_100</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" t="n">
+        <v>5170</v>
+      </c>
+      <c r="D23" t="n">
+        <v>5170</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>959</v>
+      </c>
+      <c r="G23" t="n">
+        <v>81.45</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>sao2f2_100</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>10</v>
+      </c>
+      <c r="C24" t="n">
+        <v>8260</v>
+      </c>
+      <c r="D24" t="n">
+        <v>8260</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1282</v>
+      </c>
+      <c r="G24" t="n">
+        <v>84.48</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>sao2f3_100</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C25" t="n">
+        <v>8391</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3639</v>
+      </c>
+      <c r="E25" t="n">
+        <v>56.63</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2293</v>
+      </c>
+      <c r="G25" t="n">
+        <v>72.67</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>sao2f4_100</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>10</v>
+      </c>
+      <c r="C26" t="n">
+        <v>10813</v>
+      </c>
+      <c r="D26" t="n">
+        <v>7360</v>
+      </c>
+      <c r="E26" t="n">
+        <v>31.93</v>
+      </c>
+      <c r="F26" t="n">
+        <v>3514</v>
+      </c>
+      <c r="G26" t="n">
+        <v>67.5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>sym10_d_100</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>10</v>
+      </c>
+      <c r="C27" t="n">
+        <v>51205</v>
+      </c>
+      <c r="D27" t="n">
+        <v>36281</v>
+      </c>
+      <c r="E27" t="n">
+        <v>29.15</v>
+      </c>
+      <c r="F27" t="n">
+        <v>8689</v>
+      </c>
+      <c r="G27" t="n">
+        <v>83.03</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>f_100_200-0</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>100</v>
+      </c>
+      <c r="C28" t="n">
+        <v>11983160</v>
+      </c>
+      <c r="D28" t="n">
+        <v>4061924</v>
+      </c>
+      <c r="E28" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2497516</v>
+      </c>
+      <c r="G28" t="n">
+        <v>79.16</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>f_100_200-1</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>100</v>
+      </c>
+      <c r="C29" t="n">
+        <v>11966928</v>
+      </c>
+      <c r="D29" t="n">
+        <v>3974990</v>
+      </c>
+      <c r="E29" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2020825</v>
+      </c>
+      <c r="G29" t="n">
+        <v>83.11</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>f_100_200-2</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>100</v>
+      </c>
+      <c r="C30" t="n">
+        <v>12010942</v>
+      </c>
+      <c r="D30" t="n">
+        <v>3963708</v>
+      </c>
+      <c r="E30" t="n">
+        <v>67</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2000572</v>
+      </c>
+      <c r="G30" t="n">
+        <v>83.34</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>f_100_200-3</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>100</v>
+      </c>
+      <c r="C31" t="n">
+        <v>11933054</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3973941</v>
+      </c>
+      <c r="E31" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2427255</v>
+      </c>
+      <c r="G31" t="n">
+        <v>79.66</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>f_100_200-4</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>100</v>
+      </c>
+      <c r="C32" t="n">
+        <v>12006782</v>
+      </c>
+      <c r="D32" t="n">
+        <v>3937994</v>
+      </c>
+      <c r="E32" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2397640</v>
+      </c>
+      <c r="G32" t="n">
+        <v>80.03</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>f_100_400-0</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>100</v>
+      </c>
+      <c r="C33" t="n">
+        <v>24006252</v>
+      </c>
+      <c r="D33" t="n">
+        <v>7950068</v>
+      </c>
+      <c r="E33" t="n">
+        <v>66.88</v>
+      </c>
+      <c r="F33" t="n">
+        <v>4553809</v>
+      </c>
+      <c r="G33" t="n">
+        <v>81.03</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>f_100_400-1</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>100</v>
+      </c>
+      <c r="C34" t="n">
+        <v>24211430</v>
+      </c>
+      <c r="D34" t="n">
+        <v>8217988</v>
+      </c>
+      <c r="E34" t="n">
+        <v>66.06</v>
+      </c>
+      <c r="F34" t="n">
+        <v>4580061</v>
+      </c>
+      <c r="G34" t="n">
+        <v>81.08</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>f_100_400-2</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>100</v>
+      </c>
+      <c r="C35" t="n">
+        <v>24161902</v>
+      </c>
+      <c r="D35" t="n">
+        <v>8121575</v>
+      </c>
+      <c r="E35" t="n">
+        <v>66.39</v>
+      </c>
+      <c r="F35" t="n">
+        <v>4703118</v>
+      </c>
+      <c r="G35" t="n">
+        <v>80.53</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>f_100_400-3</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>100</v>
+      </c>
+      <c r="C36" t="n">
+        <v>24012388</v>
+      </c>
+      <c r="D36" t="n">
+        <v>8033179</v>
+      </c>
+      <c r="E36" t="n">
+        <v>66.55</v>
+      </c>
+      <c r="F36" t="n">
+        <v>4634820</v>
+      </c>
+      <c r="G36" t="n">
+        <v>80.7</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>f_100_600-0</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>100</v>
+      </c>
+      <c r="C37" t="n">
+        <v>35952736</v>
+      </c>
+      <c r="D37" t="n">
+        <v>11848104</v>
+      </c>
+      <c r="E37" t="n">
+        <v>67.05</v>
+      </c>
+      <c r="F37" t="n">
+        <v>7085715</v>
+      </c>
+      <c r="G37" t="n">
+        <v>80.29000000000001</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>f_100_600-1</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>100</v>
+      </c>
+      <c r="C38" t="n">
+        <v>35986554</v>
+      </c>
+      <c r="D38" t="n">
+        <v>11674670</v>
+      </c>
+      <c r="E38" t="n">
+        <v>67.56</v>
+      </c>
+      <c r="F38" t="n">
+        <v>7008318</v>
+      </c>
+      <c r="G38" t="n">
+        <v>80.53</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>f_100_600-2</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>100</v>
+      </c>
+      <c r="C39" t="n">
+        <v>35999290</v>
+      </c>
+      <c r="D39" t="n">
+        <v>12064490</v>
+      </c>
+      <c r="E39" t="n">
+        <v>66.48999999999999</v>
+      </c>
+      <c r="F39" t="n">
+        <v>7182698</v>
+      </c>
+      <c r="G39" t="n">
+        <v>80.05</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>f_100_600-3</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>100</v>
+      </c>
+      <c r="C40" t="n">
+        <v>36082960</v>
+      </c>
+      <c r="D40" t="n">
+        <v>11976861</v>
+      </c>
+      <c r="E40" t="n">
+        <v>66.81</v>
+      </c>
+      <c r="F40" t="n">
+        <v>7225282</v>
+      </c>
+      <c r="G40" t="n">
+        <v>79.98</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>f_100_600-4</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>100</v>
+      </c>
+      <c r="C41" t="n">
+        <v>36081916</v>
+      </c>
+      <c r="D41" t="n">
+        <v>11934142</v>
+      </c>
+      <c r="E41" t="n">
+        <v>66.92</v>
+      </c>
+      <c r="F41" t="n">
+        <v>7168509</v>
+      </c>
+      <c r="G41" t="n">
+        <v>80.13</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>t481_d_100</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>16</v>
+      </c>
+      <c r="C42" t="n">
+        <v>293</v>
+      </c>
+      <c r="D42" t="n">
+        <v>185</v>
+      </c>
+      <c r="E42" t="n">
+        <v>36.86</v>
+      </c>
+      <c r="F42" t="n">
+        <v>91</v>
+      </c>
+      <c r="G42" t="n">
+        <v>68.94</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>xor5_d_100</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>5</v>
+      </c>
+      <c r="C43" t="n">
+        <v>13</v>
+      </c>
+      <c r="D43" t="n">
+        <v>13</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>13</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>xor8</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>8</v>
+      </c>
+      <c r="C44" t="n">
+        <v>279</v>
+      </c>
+      <c r="D44" t="n">
+        <v>148</v>
+      </c>
+      <c r="E44" t="n">
+        <v>46.95</v>
+      </c>
+      <c r="F44" t="n">
+        <v>148</v>
+      </c>
+      <c r="G44" t="n">
+        <v>46.95</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>z42</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>7</v>
+      </c>
+      <c r="C45" t="n">
+        <v>635</v>
+      </c>
+      <c r="D45" t="n">
+        <v>385</v>
+      </c>
+      <c r="E45" t="n">
+        <v>39.37</v>
+      </c>
+      <c r="F45" t="n">
+        <v>182</v>
+      </c>
+      <c r="G45" t="n">
+        <v>71.34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Function</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Inputs</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ESOP T</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>EOSOPS T</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>EOSOPS T Saving (%)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Final T</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Final T Saving (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>6sym</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>6</v>
       </c>
       <c r="C2" t="n">
         <v>288</v>
       </c>
       <c r="D2" t="n">
-        <v>603</v>
+        <v>224</v>
       </c>
       <c r="E2" t="n">
-        <v>224</v>
+        <v>22.22</v>
       </c>
       <c r="F2" t="n">
-        <v>29.64</v>
+        <v>96</v>
       </c>
       <c r="G2" t="n">
-        <v>207</v>
-      </c>
-      <c r="H2" t="n">
-        <v>96</v>
-      </c>
-      <c r="I2" t="n">
-        <v>75.84999999999999</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="3">
@@ -513,28 +1649,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>21212</v>
+        <v>9</v>
       </c>
       <c r="C3" t="n">
         <v>2200</v>
       </c>
       <c r="D3" t="n">
-        <v>12524</v>
+        <v>1672</v>
       </c>
       <c r="E3" t="n">
-        <v>1672</v>
+        <v>24</v>
       </c>
       <c r="F3" t="n">
-        <v>40.96</v>
+        <v>880</v>
       </c>
       <c r="G3" t="n">
-        <v>3519</v>
-      </c>
-      <c r="H3" t="n">
-        <v>880</v>
-      </c>
-      <c r="I3" t="n">
-        <v>83.41</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -544,28 +1674,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>141</v>
+        <v>7</v>
       </c>
       <c r="C4" t="n">
         <v>56</v>
       </c>
       <c r="D4" t="n">
-        <v>114</v>
+        <v>40</v>
       </c>
       <c r="E4" t="n">
-        <v>40</v>
+        <v>28.57</v>
       </c>
       <c r="F4" t="n">
-        <v>19.15</v>
+        <v>8</v>
       </c>
       <c r="G4" t="n">
-        <v>43</v>
-      </c>
-      <c r="H4" t="n">
-        <v>8</v>
-      </c>
-      <c r="I4" t="n">
-        <v>69.5</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -575,28 +1699,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>68</v>
+        <v>7</v>
       </c>
       <c r="C5" t="n">
         <v>32</v>
       </c>
       <c r="D5" t="n">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="E5" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G5" t="n">
-        <v>45</v>
-      </c>
-      <c r="H5" t="n">
-        <v>16</v>
-      </c>
-      <c r="I5" t="n">
-        <v>33.82</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -606,28 +1724,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>68</v>
+        <v>5</v>
       </c>
       <c r="C6" t="n">
         <v>32</v>
       </c>
       <c r="D6" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>67.65000000000001</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>22</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>67.65000000000001</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -637,13 +1749,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -652,12 +1764,6 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -668,28 +1774,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
         <v>16</v>
       </c>
       <c r="D8" t="n">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="E8" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G8" t="n">
-        <v>24</v>
-      </c>
-      <c r="H8" t="n">
-        <v>8</v>
-      </c>
-      <c r="I8" t="n">
-        <v>38.46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
@@ -699,28 +1799,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13108</v>
+        <v>9</v>
       </c>
       <c r="C9" t="n">
         <v>1784</v>
       </c>
       <c r="D9" t="n">
-        <v>7680</v>
+        <v>1272</v>
       </c>
       <c r="E9" t="n">
-        <v>1272</v>
+        <v>28.7</v>
       </c>
       <c r="F9" t="n">
-        <v>41.41</v>
+        <v>696</v>
       </c>
       <c r="G9" t="n">
-        <v>2464</v>
-      </c>
-      <c r="H9" t="n">
-        <v>696</v>
-      </c>
-      <c r="I9" t="n">
-        <v>81.2</v>
+        <v>60.99</v>
       </c>
     </row>
     <row r="10">
@@ -730,28 +1824,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14378</v>
+        <v>9</v>
       </c>
       <c r="C10" t="n">
         <v>1752</v>
       </c>
       <c r="D10" t="n">
-        <v>12322</v>
+        <v>1560</v>
       </c>
       <c r="E10" t="n">
-        <v>1560</v>
+        <v>10.96</v>
       </c>
       <c r="F10" t="n">
-        <v>14.3</v>
+        <v>664</v>
       </c>
       <c r="G10" t="n">
-        <v>2487</v>
-      </c>
-      <c r="H10" t="n">
-        <v>664</v>
-      </c>
-      <c r="I10" t="n">
-        <v>82.7</v>
+        <v>62.1</v>
       </c>
     </row>
     <row r="11">
@@ -761,28 +1849,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1239</v>
+        <v>8</v>
       </c>
       <c r="C11" t="n">
         <v>216</v>
       </c>
       <c r="D11" t="n">
-        <v>1239</v>
+        <v>216</v>
       </c>
       <c r="E11" t="n">
-        <v>216</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="G11" t="n">
-        <v>230</v>
-      </c>
-      <c r="H11" t="n">
-        <v>80</v>
-      </c>
-      <c r="I11" t="n">
-        <v>81.44</v>
+        <v>62.96</v>
       </c>
     </row>
     <row r="12">
@@ -792,28 +1874,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>683</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
         <v>128</v>
       </c>
       <c r="D12" t="n">
-        <v>683</v>
+        <v>128</v>
       </c>
       <c r="E12" t="n">
-        <v>128</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="G12" t="n">
-        <v>161</v>
-      </c>
-      <c r="H12" t="n">
-        <v>48</v>
-      </c>
-      <c r="I12" t="n">
-        <v>76.43000000000001</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="13">
@@ -823,28 +1899,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>185</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
         <v>80</v>
       </c>
       <c r="D13" t="n">
-        <v>75</v>
+        <v>32</v>
       </c>
       <c r="E13" t="n">
+        <v>60</v>
+      </c>
+      <c r="F13" t="n">
         <v>32</v>
       </c>
-      <c r="F13" t="n">
-        <v>59.46</v>
-      </c>
       <c r="G13" t="n">
-        <v>75</v>
-      </c>
-      <c r="H13" t="n">
-        <v>32</v>
-      </c>
-      <c r="I13" t="n">
-        <v>59.46</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14">
@@ -854,28 +1924,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>88</v>
+        <v>5</v>
       </c>
       <c r="C14" t="n">
         <v>32</v>
       </c>
       <c r="D14" t="n">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="E14" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G14" t="n">
-        <v>47</v>
-      </c>
-      <c r="H14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I14" t="n">
-        <v>46.59</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15">
@@ -885,13 +1949,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -900,12 +1964,6 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>13</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -916,28 +1974,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>211</v>
+        <v>7</v>
       </c>
       <c r="C16" t="n">
         <v>96</v>
       </c>
       <c r="D16" t="n">
-        <v>211</v>
+        <v>96</v>
       </c>
       <c r="E16" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G16" t="n">
-        <v>106</v>
-      </c>
-      <c r="H16" t="n">
-        <v>8</v>
-      </c>
-      <c r="I16" t="n">
-        <v>49.76</v>
+        <v>91.67</v>
       </c>
     </row>
     <row r="17">
@@ -947,13 +1999,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -962,12 +2014,6 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>19</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -978,28 +2024,22 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1341</v>
+        <v>7</v>
       </c>
       <c r="C18" t="n">
         <v>456</v>
       </c>
       <c r="D18" t="n">
-        <v>1318</v>
+        <v>440</v>
       </c>
       <c r="E18" t="n">
-        <v>440</v>
+        <v>3.51</v>
       </c>
       <c r="F18" t="n">
-        <v>1.72</v>
+        <v>120</v>
       </c>
       <c r="G18" t="n">
-        <v>339</v>
-      </c>
-      <c r="H18" t="n">
-        <v>120</v>
-      </c>
-      <c r="I18" t="n">
-        <v>74.72</v>
+        <v>73.68000000000001</v>
       </c>
     </row>
     <row r="19">
@@ -1009,28 +2049,22 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>277</v>
+        <v>8</v>
       </c>
       <c r="C19" t="n">
         <v>112</v>
       </c>
       <c r="D19" t="n">
-        <v>277</v>
+        <v>112</v>
       </c>
       <c r="E19" t="n">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>127</v>
-      </c>
-      <c r="H19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I19" t="n">
-        <v>54.15</v>
+        <v>92.86</v>
       </c>
     </row>
     <row r="20">
@@ -1040,13 +2074,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -1055,12 +2089,6 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>24</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1071,27 +2099,21 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>509</v>
+        <v>8</v>
       </c>
       <c r="C21" t="n">
         <v>48</v>
       </c>
       <c r="D21" t="n">
-        <v>509</v>
+        <v>48</v>
       </c>
       <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
         <v>48</v>
       </c>
-      <c r="F21" t="n">
-        <v>0</v>
-      </c>
       <c r="G21" t="n">
-        <v>509</v>
-      </c>
-      <c r="H21" t="n">
-        <v>48</v>
-      </c>
-      <c r="I21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1102,28 +2124,22 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4696</v>
+        <v>8</v>
       </c>
       <c r="C22" t="n">
         <v>1016</v>
       </c>
       <c r="D22" t="n">
-        <v>2898</v>
+        <v>808</v>
       </c>
       <c r="E22" t="n">
-        <v>808</v>
+        <v>20.47</v>
       </c>
       <c r="F22" t="n">
-        <v>38.29</v>
+        <v>360</v>
       </c>
       <c r="G22" t="n">
-        <v>910</v>
-      </c>
-      <c r="H22" t="n">
-        <v>360</v>
-      </c>
-      <c r="I22" t="n">
-        <v>80.62</v>
+        <v>64.56999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1133,28 +2149,22 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5170</v>
+        <v>10</v>
       </c>
       <c r="C23" t="n">
         <v>480</v>
       </c>
       <c r="D23" t="n">
-        <v>5170</v>
+        <v>480</v>
       </c>
       <c r="E23" t="n">
-        <v>480</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="G23" t="n">
-        <v>959</v>
-      </c>
-      <c r="H23" t="n">
-        <v>208</v>
-      </c>
-      <c r="I23" t="n">
-        <v>81.45</v>
+        <v>56.67</v>
       </c>
     </row>
     <row r="24">
@@ -1164,28 +2174,22 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8260</v>
+        <v>10</v>
       </c>
       <c r="C24" t="n">
         <v>608</v>
       </c>
       <c r="D24" t="n">
-        <v>8260</v>
+        <v>608</v>
       </c>
       <c r="E24" t="n">
-        <v>608</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="G24" t="n">
-        <v>1282</v>
-      </c>
-      <c r="H24" t="n">
-        <v>240</v>
-      </c>
-      <c r="I24" t="n">
-        <v>84.48</v>
+        <v>60.53</v>
       </c>
     </row>
     <row r="25">
@@ -1195,28 +2199,22 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>8391</v>
+        <v>10</v>
       </c>
       <c r="C25" t="n">
         <v>568</v>
       </c>
       <c r="D25" t="n">
-        <v>3639</v>
+        <v>392</v>
       </c>
       <c r="E25" t="n">
-        <v>392</v>
+        <v>30.99</v>
       </c>
       <c r="F25" t="n">
-        <v>56.63</v>
+        <v>272</v>
       </c>
       <c r="G25" t="n">
-        <v>2293</v>
-      </c>
-      <c r="H25" t="n">
-        <v>272</v>
-      </c>
-      <c r="I25" t="n">
-        <v>72.67</v>
+        <v>52.11</v>
       </c>
     </row>
     <row r="26">
@@ -1226,28 +2224,22 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>10813</v>
+        <v>10</v>
       </c>
       <c r="C26" t="n">
         <v>536</v>
       </c>
       <c r="D26" t="n">
-        <v>7360</v>
+        <v>408</v>
       </c>
       <c r="E26" t="n">
-        <v>408</v>
+        <v>23.88</v>
       </c>
       <c r="F26" t="n">
-        <v>31.93</v>
+        <v>280</v>
       </c>
       <c r="G26" t="n">
-        <v>3514</v>
-      </c>
-      <c r="H26" t="n">
-        <v>280</v>
-      </c>
-      <c r="I26" t="n">
-        <v>67.5</v>
+        <v>47.76</v>
       </c>
     </row>
     <row r="27">
@@ -1257,28 +2249,22 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>51205</v>
+        <v>10</v>
       </c>
       <c r="C27" t="n">
         <v>3880</v>
       </c>
       <c r="D27" t="n">
-        <v>36281</v>
+        <v>3216</v>
       </c>
       <c r="E27" t="n">
-        <v>3216</v>
+        <v>17.11</v>
       </c>
       <c r="F27" t="n">
-        <v>29.15</v>
+        <v>1552</v>
       </c>
       <c r="G27" t="n">
-        <v>8689</v>
-      </c>
-      <c r="H27" t="n">
-        <v>1552</v>
-      </c>
-      <c r="I27" t="n">
-        <v>83.03</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28">
@@ -1288,28 +2274,22 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>11983160</v>
+        <v>100</v>
       </c>
       <c r="C28" t="n">
         <v>103120</v>
       </c>
       <c r="D28" t="n">
-        <v>4061924</v>
+        <v>41328</v>
       </c>
       <c r="E28" t="n">
-        <v>41328</v>
+        <v>59.92</v>
       </c>
       <c r="F28" t="n">
-        <v>66.09999999999999</v>
+        <v>37752</v>
       </c>
       <c r="G28" t="n">
-        <v>2497516</v>
-      </c>
-      <c r="H28" t="n">
-        <v>37752</v>
-      </c>
-      <c r="I28" t="n">
-        <v>79.16</v>
+        <v>63.39</v>
       </c>
     </row>
     <row r="29">
@@ -1319,28 +2299,22 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>11966928</v>
+        <v>100</v>
       </c>
       <c r="C29" t="n">
         <v>102992</v>
       </c>
       <c r="D29" t="n">
-        <v>3974990</v>
+        <v>40616</v>
       </c>
       <c r="E29" t="n">
-        <v>40616</v>
+        <v>60.56</v>
       </c>
       <c r="F29" t="n">
-        <v>66.78</v>
+        <v>30432</v>
       </c>
       <c r="G29" t="n">
-        <v>2020825</v>
-      </c>
-      <c r="H29" t="n">
-        <v>30432</v>
-      </c>
-      <c r="I29" t="n">
-        <v>83.11</v>
+        <v>70.45</v>
       </c>
     </row>
     <row r="30">
@@ -1350,28 +2324,22 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>12010942</v>
+        <v>100</v>
       </c>
       <c r="C30" t="n">
         <v>103336</v>
       </c>
       <c r="D30" t="n">
-        <v>3963708</v>
+        <v>40544</v>
       </c>
       <c r="E30" t="n">
-        <v>40544</v>
+        <v>60.76</v>
       </c>
       <c r="F30" t="n">
-        <v>67</v>
+        <v>30152</v>
       </c>
       <c r="G30" t="n">
-        <v>2000572</v>
-      </c>
-      <c r="H30" t="n">
-        <v>30152</v>
-      </c>
-      <c r="I30" t="n">
-        <v>83.34</v>
+        <v>70.81999999999999</v>
       </c>
     </row>
     <row r="31">
@@ -1381,28 +2349,22 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>11933054</v>
+        <v>100</v>
       </c>
       <c r="C31" t="n">
         <v>102728</v>
       </c>
       <c r="D31" t="n">
-        <v>3973941</v>
+        <v>40640</v>
       </c>
       <c r="E31" t="n">
-        <v>40640</v>
+        <v>60.44</v>
       </c>
       <c r="F31" t="n">
-        <v>66.7</v>
+        <v>36976</v>
       </c>
       <c r="G31" t="n">
-        <v>2427255</v>
-      </c>
-      <c r="H31" t="n">
-        <v>36976</v>
-      </c>
-      <c r="I31" t="n">
-        <v>79.66</v>
+        <v>64.01000000000001</v>
       </c>
     </row>
     <row r="32">
@@ -1412,28 +2374,22 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>12006782</v>
+        <v>100</v>
       </c>
       <c r="C32" t="n">
         <v>103304</v>
       </c>
       <c r="D32" t="n">
-        <v>3937994</v>
+        <v>40360</v>
       </c>
       <c r="E32" t="n">
-        <v>40360</v>
+        <v>60.93</v>
       </c>
       <c r="F32" t="n">
-        <v>67.2</v>
+        <v>36848</v>
       </c>
       <c r="G32" t="n">
-        <v>2397640</v>
-      </c>
-      <c r="H32" t="n">
-        <v>36848</v>
-      </c>
-      <c r="I32" t="n">
-        <v>80.03</v>
+        <v>64.33</v>
       </c>
     </row>
     <row r="33">
@@ -1443,28 +2399,22 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>24006252</v>
+        <v>100</v>
       </c>
       <c r="C33" t="n">
         <v>206552</v>
       </c>
       <c r="D33" t="n">
-        <v>7950068</v>
+        <v>81264</v>
       </c>
       <c r="E33" t="n">
-        <v>81264</v>
+        <v>60.66</v>
       </c>
       <c r="F33" t="n">
-        <v>66.88</v>
+        <v>68568</v>
       </c>
       <c r="G33" t="n">
-        <v>4553809</v>
-      </c>
-      <c r="H33" t="n">
-        <v>68568</v>
-      </c>
-      <c r="I33" t="n">
-        <v>81.03</v>
+        <v>66.8</v>
       </c>
     </row>
     <row r="34">
@@ -1474,28 +2424,22 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>24211430</v>
+        <v>100</v>
       </c>
       <c r="C34" t="n">
         <v>208152</v>
       </c>
       <c r="D34" t="n">
-        <v>8217988</v>
+        <v>83392</v>
       </c>
       <c r="E34" t="n">
-        <v>83392</v>
+        <v>59.94</v>
       </c>
       <c r="F34" t="n">
-        <v>66.06</v>
+        <v>68600</v>
       </c>
       <c r="G34" t="n">
-        <v>4580061</v>
-      </c>
-      <c r="H34" t="n">
-        <v>68600</v>
-      </c>
-      <c r="I34" t="n">
-        <v>81.08</v>
+        <v>67.04000000000001</v>
       </c>
     </row>
     <row r="35">
@@ -1505,28 +2449,22 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>24161902</v>
+        <v>100</v>
       </c>
       <c r="C35" t="n">
         <v>207768</v>
       </c>
       <c r="D35" t="n">
-        <v>8121575</v>
+        <v>82640</v>
       </c>
       <c r="E35" t="n">
-        <v>82640</v>
+        <v>60.22</v>
       </c>
       <c r="F35" t="n">
-        <v>66.39</v>
+        <v>69896</v>
       </c>
       <c r="G35" t="n">
-        <v>4703118</v>
-      </c>
-      <c r="H35" t="n">
-        <v>69896</v>
-      </c>
-      <c r="I35" t="n">
-        <v>80.53</v>
+        <v>66.36</v>
       </c>
     </row>
     <row r="36">
@@ -1536,28 +2474,22 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>24012388</v>
+        <v>100</v>
       </c>
       <c r="C36" t="n">
         <v>206600</v>
       </c>
       <c r="D36" t="n">
-        <v>8033179</v>
+        <v>81840</v>
       </c>
       <c r="E36" t="n">
-        <v>81840</v>
+        <v>60.39</v>
       </c>
       <c r="F36" t="n">
-        <v>66.55</v>
+        <v>69176</v>
       </c>
       <c r="G36" t="n">
-        <v>4634820</v>
-      </c>
-      <c r="H36" t="n">
-        <v>69176</v>
-      </c>
-      <c r="I36" t="n">
-        <v>80.7</v>
+        <v>66.52</v>
       </c>
     </row>
     <row r="37">
@@ -1567,28 +2499,22 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>35952736</v>
+        <v>100</v>
       </c>
       <c r="C37" t="n">
         <v>309384</v>
       </c>
       <c r="D37" t="n">
-        <v>11848104</v>
+        <v>121312</v>
       </c>
       <c r="E37" t="n">
-        <v>121312</v>
+        <v>60.79</v>
       </c>
       <c r="F37" t="n">
-        <v>67.05</v>
+        <v>106272</v>
       </c>
       <c r="G37" t="n">
-        <v>7085715</v>
-      </c>
-      <c r="H37" t="n">
-        <v>106272</v>
-      </c>
-      <c r="I37" t="n">
-        <v>80.29000000000001</v>
+        <v>65.65000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -1598,28 +2524,22 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>35986554</v>
+        <v>100</v>
       </c>
       <c r="C38" t="n">
         <v>309648</v>
       </c>
       <c r="D38" t="n">
-        <v>11674670</v>
+        <v>119976</v>
       </c>
       <c r="E38" t="n">
-        <v>119976</v>
+        <v>61.25</v>
       </c>
       <c r="F38" t="n">
-        <v>67.56</v>
+        <v>105576</v>
       </c>
       <c r="G38" t="n">
-        <v>7008318</v>
-      </c>
-      <c r="H38" t="n">
-        <v>105576</v>
-      </c>
-      <c r="I38" t="n">
-        <v>80.53</v>
+        <v>65.90000000000001</v>
       </c>
     </row>
     <row r="39">
@@ -1629,28 +2549,22 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>35999290</v>
+        <v>100</v>
       </c>
       <c r="C39" t="n">
         <v>309744</v>
       </c>
       <c r="D39" t="n">
-        <v>12064490</v>
+        <v>122984</v>
       </c>
       <c r="E39" t="n">
-        <v>122984</v>
+        <v>60.29</v>
       </c>
       <c r="F39" t="n">
-        <v>66.48999999999999</v>
+        <v>107440</v>
       </c>
       <c r="G39" t="n">
-        <v>7182698</v>
-      </c>
-      <c r="H39" t="n">
-        <v>107440</v>
-      </c>
-      <c r="I39" t="n">
-        <v>80.05</v>
+        <v>65.31</v>
       </c>
     </row>
     <row r="40">
@@ -1660,28 +2574,22 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>36082960</v>
+        <v>100</v>
       </c>
       <c r="C40" t="n">
         <v>310400</v>
       </c>
       <c r="D40" t="n">
-        <v>11976861</v>
+        <v>122336</v>
       </c>
       <c r="E40" t="n">
-        <v>122336</v>
+        <v>60.59</v>
       </c>
       <c r="F40" t="n">
-        <v>66.81</v>
+        <v>107680</v>
       </c>
       <c r="G40" t="n">
-        <v>7225282</v>
-      </c>
-      <c r="H40" t="n">
-        <v>107680</v>
-      </c>
-      <c r="I40" t="n">
-        <v>79.98</v>
+        <v>65.31</v>
       </c>
     </row>
     <row r="41">
@@ -1691,28 +2599,22 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>36081916</v>
+        <v>100</v>
       </c>
       <c r="C41" t="n">
         <v>310392</v>
       </c>
       <c r="D41" t="n">
-        <v>11934142</v>
+        <v>122000</v>
       </c>
       <c r="E41" t="n">
-        <v>122000</v>
+        <v>60.69</v>
       </c>
       <c r="F41" t="n">
-        <v>66.92</v>
+        <v>107168</v>
       </c>
       <c r="G41" t="n">
-        <v>7168509</v>
-      </c>
-      <c r="H41" t="n">
-        <v>107168</v>
-      </c>
-      <c r="I41" t="n">
-        <v>80.13</v>
+        <v>65.47</v>
       </c>
     </row>
     <row r="42">
@@ -1722,28 +2624,22 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>293</v>
+        <v>16</v>
       </c>
       <c r="C42" t="n">
         <v>128</v>
       </c>
       <c r="D42" t="n">
-        <v>185</v>
+        <v>64</v>
       </c>
       <c r="E42" t="n">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="F42" t="n">
-        <v>36.86</v>
+        <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>91</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" t="n">
-        <v>68.94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43">
@@ -1753,13 +2649,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C43" t="n">
         <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
@@ -1768,12 +2664,6 @@
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>13</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1784,28 +2674,22 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>279</v>
+        <v>8</v>
       </c>
       <c r="C44" t="n">
         <v>40</v>
       </c>
       <c r="D44" t="n">
-        <v>148</v>
+        <v>32</v>
       </c>
       <c r="E44" t="n">
+        <v>20</v>
+      </c>
+      <c r="F44" t="n">
         <v>32</v>
       </c>
-      <c r="F44" t="n">
-        <v>46.95</v>
-      </c>
       <c r="G44" t="n">
-        <v>148</v>
-      </c>
-      <c r="H44" t="n">
-        <v>32</v>
-      </c>
-      <c r="I44" t="n">
-        <v>46.95</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45">
@@ -1815,28 +2699,22 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>635</v>
+        <v>7</v>
       </c>
       <c r="C45" t="n">
         <v>152</v>
       </c>
       <c r="D45" t="n">
-        <v>385</v>
+        <v>120</v>
       </c>
       <c r="E45" t="n">
-        <v>120</v>
+        <v>21.05</v>
       </c>
       <c r="F45" t="n">
-        <v>39.37</v>
+        <v>80</v>
       </c>
       <c r="G45" t="n">
-        <v>182</v>
-      </c>
-      <c r="H45" t="n">
-        <v>80</v>
-      </c>
-      <c r="I45" t="n">
-        <v>71.34</v>
+        <v>47.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added more benchmarks. Generated new results table. Minor change to makefile.
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,473 +469,473 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6sym</t>
+          <t>4gt10_22</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>857</v>
+        <v>36</v>
       </c>
       <c r="D2" t="n">
-        <v>603</v>
+        <v>36</v>
       </c>
       <c r="E2" t="n">
-        <v>29.64</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>207</v>
+        <v>17</v>
       </c>
       <c r="G2" t="n">
-        <v>75.84999999999999</v>
+        <v>52.78</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9sym_d_100</t>
+          <t>4mod5_8</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>21212</v>
+        <v>28</v>
       </c>
       <c r="D3" t="n">
-        <v>12524</v>
+        <v>28</v>
       </c>
       <c r="E3" t="n">
-        <v>40.96</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>3519</v>
+        <v>10</v>
       </c>
       <c r="G3" t="n">
-        <v>83.41</v>
+        <v>64.29000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>con1f1_100</t>
+          <t>6sym</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="n">
-        <v>141</v>
+        <v>857</v>
       </c>
       <c r="D4" t="n">
-        <v>114</v>
+        <v>603</v>
       </c>
       <c r="E4" t="n">
-        <v>19.15</v>
+        <v>29.64</v>
       </c>
       <c r="F4" t="n">
-        <v>43</v>
+        <v>207</v>
       </c>
       <c r="G4" t="n">
-        <v>69.5</v>
+        <v>75.84999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>con2f2_100</t>
+          <t>9sym_d_100</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>68</v>
+        <v>21212</v>
       </c>
       <c r="D5" t="n">
-        <v>68</v>
+        <v>12524</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>40.96</v>
       </c>
       <c r="F5" t="n">
-        <v>45</v>
+        <v>3519</v>
       </c>
       <c r="G5" t="n">
-        <v>33.82</v>
+        <v>83.41</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>eosops1_100</t>
+          <t>alu_9</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="D6" t="n">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="E6" t="n">
-        <v>67.65000000000001</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="G6" t="n">
-        <v>67.65000000000001</v>
+        <v>28.85</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>exam1_d_100</t>
+          <t>con1f1_100</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>141</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>114</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>19.15</v>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>69.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>exam3_d_100</t>
+          <t>con2f2_100</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="D8" t="n">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="G8" t="n">
-        <v>38.46</v>
+        <v>33.82</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>life_d_100</t>
+          <t>eosops1_100</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>13108</v>
+        <v>68</v>
       </c>
       <c r="D9" t="n">
-        <v>7680</v>
+        <v>22</v>
       </c>
       <c r="E9" t="n">
-        <v>41.41</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>2464</v>
+        <v>22</v>
       </c>
       <c r="G9" t="n">
-        <v>81.2</v>
+        <v>67.65000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>max46_d_100</t>
+          <t>exam1_d_100</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>14378</v>
+        <v>5</v>
       </c>
       <c r="D10" t="n">
-        <v>12322</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>2487</v>
+        <v>5</v>
       </c>
       <c r="G10" t="n">
-        <v>82.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>newill_d_100</t>
+          <t>exam3_d_100</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>1239</v>
+        <v>39</v>
       </c>
       <c r="D11" t="n">
-        <v>1239</v>
+        <v>39</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>230</v>
+        <v>24</v>
       </c>
       <c r="G11" t="n">
-        <v>81.44</v>
+        <v>38.46</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>newtag_d_100</t>
+          <t>life_d_100</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" t="n">
-        <v>683</v>
+        <v>13108</v>
       </c>
       <c r="D12" t="n">
-        <v>683</v>
+        <v>7680</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>41.41</v>
       </c>
       <c r="F12" t="n">
-        <v>161</v>
+        <v>2464</v>
       </c>
       <c r="G12" t="n">
-        <v>76.43000000000001</v>
+        <v>81.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>rd53f1_100</t>
+          <t>majority_176</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>185</v>
+        <v>149</v>
       </c>
       <c r="D13" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="E13" t="n">
-        <v>59.46</v>
+        <v>39.6</v>
       </c>
       <c r="F13" t="n">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="G13" t="n">
-        <v>59.46</v>
+        <v>71.14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>rd53f2_100</t>
+          <t>max46_d_100</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C14" t="n">
-        <v>88</v>
+        <v>14378</v>
       </c>
       <c r="D14" t="n">
-        <v>88</v>
+        <v>12322</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="F14" t="n">
-        <v>47</v>
+        <v>2487</v>
       </c>
       <c r="G14" t="n">
-        <v>46.59</v>
+        <v>82.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rd53f3_100</t>
+          <t>mux_185</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="C15" t="n">
-        <v>13</v>
+        <v>2064</v>
       </c>
       <c r="D15" t="n">
-        <v>13</v>
+        <v>2064</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>13</v>
+        <v>328</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>84.11</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>rd73f1_100</t>
+          <t>newill_d_100</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C16" t="n">
-        <v>211</v>
+        <v>1239</v>
       </c>
       <c r="D16" t="n">
-        <v>211</v>
+        <v>1239</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>106</v>
+        <v>230</v>
       </c>
       <c r="G16" t="n">
-        <v>49.76</v>
+        <v>81.44</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>rd73f2_100</t>
+          <t>newtag_d_100</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C17" t="n">
-        <v>19</v>
+        <v>683</v>
       </c>
       <c r="D17" t="n">
-        <v>19</v>
+        <v>683</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>19</v>
+        <v>161</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>76.43000000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>rd73f3_100</t>
+          <t>rd53f1_100</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>1341</v>
+        <v>185</v>
       </c>
       <c r="D18" t="n">
-        <v>1318</v>
+        <v>75</v>
       </c>
       <c r="E18" t="n">
-        <v>1.72</v>
+        <v>59.46</v>
       </c>
       <c r="F18" t="n">
-        <v>339</v>
+        <v>75</v>
       </c>
       <c r="G18" t="n">
-        <v>74.72</v>
+        <v>59.46</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>rd84f1_100</t>
+          <t>rd53f2_100</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>277</v>
+        <v>88</v>
       </c>
       <c r="D19" t="n">
-        <v>277</v>
+        <v>88</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>127</v>
+        <v>47</v>
       </c>
       <c r="G19" t="n">
-        <v>54.15</v>
+        <v>46.59</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>rd84f2_100</t>
+          <t>rd53f3_100</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D20" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -944,625 +944,800 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>rd84f3_100</t>
+          <t>rd73f1_100</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>509</v>
+        <v>211</v>
       </c>
       <c r="D21" t="n">
-        <v>509</v>
+        <v>211</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>509</v>
+        <v>106</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>49.76</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>rd84f4_100</t>
+          <t>rd73f2_100</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C22" t="n">
-        <v>4696</v>
+        <v>19</v>
       </c>
       <c r="D22" t="n">
-        <v>2898</v>
+        <v>19</v>
       </c>
       <c r="E22" t="n">
-        <v>38.29</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>910</v>
+        <v>19</v>
       </c>
       <c r="G22" t="n">
-        <v>80.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sao2f1_100</t>
+          <t>rd73f3_100</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>5170</v>
+        <v>1341</v>
       </c>
       <c r="D23" t="n">
-        <v>5170</v>
+        <v>1318</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1.72</v>
       </c>
       <c r="F23" t="n">
-        <v>959</v>
+        <v>339</v>
       </c>
       <c r="G23" t="n">
-        <v>81.45</v>
+        <v>74.72</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sao2f2_100</t>
+          <t>rd84f1_100</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C24" t="n">
-        <v>8260</v>
+        <v>277</v>
       </c>
       <c r="D24" t="n">
-        <v>8260</v>
+        <v>277</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>1282</v>
+        <v>127</v>
       </c>
       <c r="G24" t="n">
-        <v>84.48</v>
+        <v>54.15</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sao2f3_100</t>
+          <t>rd84f2_100</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C25" t="n">
-        <v>8391</v>
+        <v>24</v>
       </c>
       <c r="D25" t="n">
-        <v>3639</v>
+        <v>24</v>
       </c>
       <c r="E25" t="n">
-        <v>56.63</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2293</v>
+        <v>24</v>
       </c>
       <c r="G25" t="n">
-        <v>72.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sao2f4_100</t>
+          <t>rd84f3_100</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C26" t="n">
-        <v>10813</v>
+        <v>509</v>
       </c>
       <c r="D26" t="n">
-        <v>7360</v>
+        <v>509</v>
       </c>
       <c r="E26" t="n">
-        <v>31.93</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>3514</v>
+        <v>509</v>
       </c>
       <c r="G26" t="n">
-        <v>67.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sym10_d_100</t>
+          <t>rd84f4_100</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C27" t="n">
-        <v>51205</v>
+        <v>4696</v>
       </c>
       <c r="D27" t="n">
-        <v>36281</v>
+        <v>2898</v>
       </c>
       <c r="E27" t="n">
-        <v>29.15</v>
+        <v>38.29</v>
       </c>
       <c r="F27" t="n">
-        <v>8689</v>
+        <v>910</v>
       </c>
       <c r="G27" t="n">
-        <v>83.03</v>
+        <v>80.62</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>f_100_200-0</t>
+          <t>ryy6_198</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>100</v>
+        <v>16</v>
       </c>
       <c r="C28" t="n">
-        <v>11983160</v>
+        <v>61084</v>
       </c>
       <c r="D28" t="n">
-        <v>4061924</v>
+        <v>20064</v>
       </c>
       <c r="E28" t="n">
-        <v>66.09999999999999</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="F28" t="n">
-        <v>2497516</v>
+        <v>20064</v>
       </c>
       <c r="G28" t="n">
-        <v>79.16</v>
+        <v>67.15000000000001</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>f_100_200-1</t>
+          <t>sao2f1_100</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C29" t="n">
-        <v>11966928</v>
+        <v>5170</v>
       </c>
       <c r="D29" t="n">
-        <v>3974990</v>
+        <v>5170</v>
       </c>
       <c r="E29" t="n">
-        <v>66.78</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>2020825</v>
+        <v>959</v>
       </c>
       <c r="G29" t="n">
-        <v>83.11</v>
+        <v>81.45</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>f_100_200-2</t>
+          <t>sao2f2_100</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C30" t="n">
-        <v>12010942</v>
+        <v>8260</v>
       </c>
       <c r="D30" t="n">
-        <v>3963708</v>
+        <v>8260</v>
       </c>
       <c r="E30" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>2000572</v>
+        <v>1282</v>
       </c>
       <c r="G30" t="n">
-        <v>83.34</v>
+        <v>84.48</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>f_100_200-3</t>
+          <t>sao2f3_100</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C31" t="n">
-        <v>11933054</v>
+        <v>8391</v>
       </c>
       <c r="D31" t="n">
-        <v>3973941</v>
+        <v>3639</v>
       </c>
       <c r="E31" t="n">
-        <v>66.7</v>
+        <v>56.63</v>
       </c>
       <c r="F31" t="n">
-        <v>2427255</v>
+        <v>2293</v>
       </c>
       <c r="G31" t="n">
-        <v>79.66</v>
+        <v>72.67</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>f_100_200-4</t>
+          <t>sao2f4_100</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C32" t="n">
-        <v>12006782</v>
+        <v>10813</v>
       </c>
       <c r="D32" t="n">
-        <v>3937994</v>
+        <v>7360</v>
       </c>
       <c r="E32" t="n">
-        <v>67.2</v>
+        <v>31.93</v>
       </c>
       <c r="F32" t="n">
-        <v>2397640</v>
+        <v>3514</v>
       </c>
       <c r="G32" t="n">
-        <v>80.03</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>f_100_400-0</t>
+          <t>sf_232</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="C33" t="n">
-        <v>24006252</v>
+        <v>40</v>
       </c>
       <c r="D33" t="n">
-        <v>7950068</v>
+        <v>33</v>
       </c>
       <c r="E33" t="n">
-        <v>66.88</v>
+        <v>17.5</v>
       </c>
       <c r="F33" t="n">
-        <v>4553809</v>
+        <v>33</v>
       </c>
       <c r="G33" t="n">
-        <v>81.03</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>f_100_400-1</t>
+          <t>sym10_d_100</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C34" t="n">
-        <v>24211430</v>
+        <v>51205</v>
       </c>
       <c r="D34" t="n">
-        <v>8217988</v>
+        <v>36281</v>
       </c>
       <c r="E34" t="n">
-        <v>66.06</v>
+        <v>29.15</v>
       </c>
       <c r="F34" t="n">
-        <v>4580061</v>
+        <v>8689</v>
       </c>
       <c r="G34" t="n">
-        <v>81.08</v>
+        <v>83.03</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>f_100_400-2</t>
+          <t>f_100_200-0</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>100</v>
       </c>
       <c r="C35" t="n">
-        <v>24161902</v>
+        <v>11983160</v>
       </c>
       <c r="D35" t="n">
-        <v>8121575</v>
+        <v>4061924</v>
       </c>
       <c r="E35" t="n">
-        <v>66.39</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="F35" t="n">
-        <v>4703118</v>
+        <v>2497516</v>
       </c>
       <c r="G35" t="n">
-        <v>80.53</v>
+        <v>79.16</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>f_100_400-3</t>
+          <t>f_100_200-1</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>100</v>
       </c>
       <c r="C36" t="n">
-        <v>24012388</v>
+        <v>11966928</v>
       </c>
       <c r="D36" t="n">
-        <v>8033179</v>
+        <v>3974990</v>
       </c>
       <c r="E36" t="n">
-        <v>66.55</v>
+        <v>66.78</v>
       </c>
       <c r="F36" t="n">
-        <v>4634820</v>
+        <v>2020825</v>
       </c>
       <c r="G36" t="n">
-        <v>80.7</v>
+        <v>83.11</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>f_100_600-0</t>
+          <t>f_100_200-2</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>100</v>
       </c>
       <c r="C37" t="n">
-        <v>35952736</v>
+        <v>12010942</v>
       </c>
       <c r="D37" t="n">
-        <v>11848104</v>
+        <v>3963708</v>
       </c>
       <c r="E37" t="n">
-        <v>67.05</v>
+        <v>67</v>
       </c>
       <c r="F37" t="n">
-        <v>7085715</v>
+        <v>2000572</v>
       </c>
       <c r="G37" t="n">
-        <v>80.29000000000001</v>
+        <v>83.34</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>f_100_600-1</t>
+          <t>f_100_200-3</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>100</v>
       </c>
       <c r="C38" t="n">
-        <v>35986554</v>
+        <v>11933054</v>
       </c>
       <c r="D38" t="n">
-        <v>11674670</v>
+        <v>3973941</v>
       </c>
       <c r="E38" t="n">
-        <v>67.56</v>
+        <v>66.7</v>
       </c>
       <c r="F38" t="n">
-        <v>7008318</v>
+        <v>2427255</v>
       </c>
       <c r="G38" t="n">
-        <v>80.53</v>
+        <v>79.66</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>f_100_600-2</t>
+          <t>f_100_200-4</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>100</v>
       </c>
       <c r="C39" t="n">
-        <v>35999290</v>
+        <v>12006782</v>
       </c>
       <c r="D39" t="n">
-        <v>12064490</v>
+        <v>3937994</v>
       </c>
       <c r="E39" t="n">
-        <v>66.48999999999999</v>
+        <v>67.2</v>
       </c>
       <c r="F39" t="n">
-        <v>7182698</v>
+        <v>2397640</v>
       </c>
       <c r="G39" t="n">
-        <v>80.05</v>
+        <v>80.03</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>f_100_600-3</t>
+          <t>f_100_400-0</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>100</v>
       </c>
       <c r="C40" t="n">
-        <v>36082960</v>
+        <v>24006252</v>
       </c>
       <c r="D40" t="n">
-        <v>11976861</v>
+        <v>7950068</v>
       </c>
       <c r="E40" t="n">
-        <v>66.81</v>
+        <v>66.88</v>
       </c>
       <c r="F40" t="n">
-        <v>7225282</v>
+        <v>4553809</v>
       </c>
       <c r="G40" t="n">
-        <v>79.98</v>
+        <v>81.03</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>f_100_600-4</t>
+          <t>f_100_400-1</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>100</v>
       </c>
       <c r="C41" t="n">
-        <v>36081916</v>
+        <v>24211430</v>
       </c>
       <c r="D41" t="n">
-        <v>11934142</v>
+        <v>8217988</v>
       </c>
       <c r="E41" t="n">
-        <v>66.92</v>
+        <v>66.06</v>
       </c>
       <c r="F41" t="n">
-        <v>7168509</v>
+        <v>4580061</v>
       </c>
       <c r="G41" t="n">
-        <v>80.13</v>
+        <v>81.08</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>t481_d_100</t>
+          <t>f_100_400-2</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="C42" t="n">
-        <v>293</v>
+        <v>24161902</v>
       </c>
       <c r="D42" t="n">
-        <v>185</v>
+        <v>8121575</v>
       </c>
       <c r="E42" t="n">
-        <v>36.86</v>
+        <v>66.39</v>
       </c>
       <c r="F42" t="n">
-        <v>91</v>
+        <v>4703118</v>
       </c>
       <c r="G42" t="n">
-        <v>68.94</v>
+        <v>80.53</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>xor5_d_100</t>
+          <t>f_100_400-3</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="C43" t="n">
-        <v>13</v>
+        <v>24012388</v>
       </c>
       <c r="D43" t="n">
-        <v>13</v>
+        <v>8033179</v>
       </c>
       <c r="E43" t="n">
-        <v>0</v>
+        <v>66.55</v>
       </c>
       <c r="F43" t="n">
-        <v>13</v>
+        <v>4634820</v>
       </c>
       <c r="G43" t="n">
-        <v>0</v>
+        <v>80.7</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>xor8</t>
+          <t>f_100_600-0</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="C44" t="n">
-        <v>279</v>
+        <v>35952736</v>
       </c>
       <c r="D44" t="n">
-        <v>148</v>
+        <v>11848104</v>
       </c>
       <c r="E44" t="n">
-        <v>46.95</v>
+        <v>67.05</v>
       </c>
       <c r="F44" t="n">
-        <v>148</v>
+        <v>7085715</v>
       </c>
       <c r="G44" t="n">
-        <v>46.95</v>
+        <v>80.29000000000001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>f_100_600-1</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>100</v>
+      </c>
+      <c r="C45" t="n">
+        <v>35986554</v>
+      </c>
+      <c r="D45" t="n">
+        <v>11674670</v>
+      </c>
+      <c r="E45" t="n">
+        <v>67.56</v>
+      </c>
+      <c r="F45" t="n">
+        <v>7008318</v>
+      </c>
+      <c r="G45" t="n">
+        <v>80.53</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>f_100_600-2</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>100</v>
+      </c>
+      <c r="C46" t="n">
+        <v>35999290</v>
+      </c>
+      <c r="D46" t="n">
+        <v>12064490</v>
+      </c>
+      <c r="E46" t="n">
+        <v>66.48999999999999</v>
+      </c>
+      <c r="F46" t="n">
+        <v>7182698</v>
+      </c>
+      <c r="G46" t="n">
+        <v>80.05</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>f_100_600-3</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>100</v>
+      </c>
+      <c r="C47" t="n">
+        <v>36082960</v>
+      </c>
+      <c r="D47" t="n">
+        <v>11976861</v>
+      </c>
+      <c r="E47" t="n">
+        <v>66.81</v>
+      </c>
+      <c r="F47" t="n">
+        <v>7225282</v>
+      </c>
+      <c r="G47" t="n">
+        <v>79.98</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>f_100_600-4</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>100</v>
+      </c>
+      <c r="C48" t="n">
+        <v>36081916</v>
+      </c>
+      <c r="D48" t="n">
+        <v>11934142</v>
+      </c>
+      <c r="E48" t="n">
+        <v>66.92</v>
+      </c>
+      <c r="F48" t="n">
+        <v>7168509</v>
+      </c>
+      <c r="G48" t="n">
+        <v>80.13</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>t481_d_100</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>16</v>
+      </c>
+      <c r="C49" t="n">
+        <v>293</v>
+      </c>
+      <c r="D49" t="n">
+        <v>185</v>
+      </c>
+      <c r="E49" t="n">
+        <v>36.86</v>
+      </c>
+      <c r="F49" t="n">
+        <v>91</v>
+      </c>
+      <c r="G49" t="n">
+        <v>68.94</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>xor5_d_100</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>5</v>
+      </c>
+      <c r="C50" t="n">
+        <v>13</v>
+      </c>
+      <c r="D50" t="n">
+        <v>13</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="n">
+        <v>13</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>xor8</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>8</v>
+      </c>
+      <c r="C51" t="n">
+        <v>279</v>
+      </c>
+      <c r="D51" t="n">
+        <v>148</v>
+      </c>
+      <c r="E51" t="n">
+        <v>46.95</v>
+      </c>
+      <c r="F51" t="n">
+        <v>148</v>
+      </c>
+      <c r="G51" t="n">
+        <v>46.95</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>z42</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B52" t="n">
         <v>7</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C52" t="n">
         <v>635</v>
       </c>
-      <c r="D45" t="n">
+      <c r="D52" t="n">
         <v>385</v>
       </c>
-      <c r="E45" t="n">
+      <c r="E52" t="n">
         <v>39.37</v>
       </c>
-      <c r="F45" t="n">
+      <c r="F52" t="n">
         <v>182</v>
       </c>
-      <c r="G45" t="n">
+      <c r="G52" t="n">
         <v>71.34</v>
       </c>
     </row>
@@ -1577,7 +1752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1620,173 +1795,173 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6sym</t>
+          <t>4gt10_22</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>288</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>224</v>
+        <v>16</v>
       </c>
       <c r="E2" t="n">
-        <v>22.22</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>96</v>
+        <v>8</v>
       </c>
       <c r="G2" t="n">
-        <v>66.67</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9sym_d_100</t>
+          <t>4mod5_8</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>2200</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>1672</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>880</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>con1f1_100</t>
+          <t>6sym</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="n">
-        <v>56</v>
+        <v>288</v>
       </c>
       <c r="D4" t="n">
-        <v>40</v>
+        <v>224</v>
       </c>
       <c r="E4" t="n">
-        <v>28.57</v>
+        <v>22.22</v>
       </c>
       <c r="F4" t="n">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="G4" t="n">
-        <v>85.70999999999999</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>con2f2_100</t>
+          <t>9sym_d_100</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>32</v>
+        <v>2200</v>
       </c>
       <c r="D5" t="n">
-        <v>32</v>
+        <v>1672</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F5" t="n">
-        <v>16</v>
+        <v>880</v>
       </c>
       <c r="G5" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>eosops1_100</t>
+          <t>alu_9</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G6" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>exam1_d_100</t>
+          <t>con1f1_100</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>28.57</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>exam3_d_100</t>
+          <t>con2f2_100</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
+        <v>32</v>
+      </c>
+      <c r="D8" t="n">
+        <v>32</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
         <v>16</v>
-      </c>
-      <c r="D8" t="n">
-        <v>16</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>8</v>
       </c>
       <c r="G8" t="n">
         <v>50</v>
@@ -1795,267 +1970,267 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>life_d_100</t>
+          <t>eosops1_100</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>1784</v>
+        <v>32</v>
       </c>
       <c r="D9" t="n">
-        <v>1272</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>28.7</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>696</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>60.99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>max46_d_100</t>
+          <t>exam1_d_100</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>1752</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>1560</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>10.96</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>664</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>62.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>newill_d_100</t>
+          <t>exam3_d_100</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
         <v>8</v>
       </c>
-      <c r="C11" t="n">
-        <v>216</v>
-      </c>
-      <c r="D11" t="n">
-        <v>216</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>80</v>
-      </c>
       <c r="G11" t="n">
-        <v>62.96</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>newtag_d_100</t>
+          <t>life_d_100</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" t="n">
-        <v>128</v>
+        <v>1784</v>
       </c>
       <c r="D12" t="n">
-        <v>128</v>
+        <v>1272</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>28.7</v>
       </c>
       <c r="F12" t="n">
-        <v>48</v>
+        <v>696</v>
       </c>
       <c r="G12" t="n">
-        <v>62.5</v>
+        <v>60.99</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>rd53f1_100</t>
+          <t>majority_176</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="D13" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E13" t="n">
-        <v>60</v>
+        <v>37.5</v>
       </c>
       <c r="F13" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G13" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>rd53f2_100</t>
+          <t>max46_d_100</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C14" t="n">
-        <v>32</v>
+        <v>1752</v>
       </c>
       <c r="D14" t="n">
-        <v>32</v>
+        <v>1560</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>10.96</v>
       </c>
       <c r="F14" t="n">
-        <v>8</v>
+        <v>664</v>
       </c>
       <c r="G14" t="n">
-        <v>75</v>
+        <v>62.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rd53f3_100</t>
+          <t>mux_185</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>rd73f1_100</t>
+          <t>newill_d_100</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C16" t="n">
-        <v>96</v>
+        <v>216</v>
       </c>
       <c r="D16" t="n">
-        <v>96</v>
+        <v>216</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="G16" t="n">
-        <v>91.67</v>
+        <v>62.96</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>rd73f2_100</t>
+          <t>newtag_d_100</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>rd73f3_100</t>
+          <t>rd53f1_100</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>456</v>
+        <v>80</v>
       </c>
       <c r="D18" t="n">
-        <v>440</v>
+        <v>32</v>
       </c>
       <c r="E18" t="n">
-        <v>3.51</v>
+        <v>60</v>
       </c>
       <c r="F18" t="n">
-        <v>120</v>
+        <v>32</v>
       </c>
       <c r="G18" t="n">
-        <v>73.68000000000001</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>rd84f1_100</t>
+          <t>rd53f2_100</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>112</v>
+        <v>32</v>
       </c>
       <c r="D19" t="n">
-        <v>112</v>
+        <v>32</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -2064,17 +2239,17 @@
         <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>92.86</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>rd84f2_100</t>
+          <t>rd53f3_100</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
@@ -2095,625 +2270,800 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>rd84f3_100</t>
+          <t>rd73f1_100</t>
         </is>
       </c>
       <c r="B21" t="n">
+        <v>7</v>
+      </c>
+      <c r="C21" t="n">
+        <v>96</v>
+      </c>
+      <c r="D21" t="n">
+        <v>96</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
         <v>8</v>
       </c>
-      <c r="C21" t="n">
-        <v>48</v>
-      </c>
-      <c r="D21" t="n">
-        <v>48</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" t="n">
-        <v>48</v>
-      </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>91.67</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>rd84f4_100</t>
+          <t>rd73f2_100</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C22" t="n">
-        <v>1016</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>808</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>20.47</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>360</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>64.56999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sao2f1_100</t>
+          <t>rd73f3_100</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>480</v>
+        <v>456</v>
       </c>
       <c r="D23" t="n">
-        <v>480</v>
+        <v>440</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>3.51</v>
       </c>
       <c r="F23" t="n">
-        <v>208</v>
+        <v>120</v>
       </c>
       <c r="G23" t="n">
-        <v>56.67</v>
+        <v>73.68000000000001</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sao2f2_100</t>
+          <t>rd84f1_100</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C24" t="n">
-        <v>608</v>
+        <v>112</v>
       </c>
       <c r="D24" t="n">
-        <v>608</v>
+        <v>112</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>240</v>
+        <v>8</v>
       </c>
       <c r="G24" t="n">
-        <v>60.53</v>
+        <v>92.86</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sao2f3_100</t>
+          <t>rd84f2_100</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C25" t="n">
-        <v>568</v>
+        <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>392</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>30.99</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>272</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>52.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sao2f4_100</t>
+          <t>rd84f3_100</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C26" t="n">
-        <v>536</v>
+        <v>48</v>
       </c>
       <c r="D26" t="n">
-        <v>408</v>
+        <v>48</v>
       </c>
       <c r="E26" t="n">
-        <v>23.88</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>280</v>
+        <v>48</v>
       </c>
       <c r="G26" t="n">
-        <v>47.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sym10_d_100</t>
+          <t>rd84f4_100</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C27" t="n">
-        <v>3880</v>
+        <v>1016</v>
       </c>
       <c r="D27" t="n">
-        <v>3216</v>
+        <v>808</v>
       </c>
       <c r="E27" t="n">
-        <v>17.11</v>
+        <v>20.47</v>
       </c>
       <c r="F27" t="n">
-        <v>1552</v>
+        <v>360</v>
       </c>
       <c r="G27" t="n">
-        <v>60</v>
+        <v>64.56999999999999</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>f_100_200-0</t>
+          <t>ryy6_198</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>100</v>
+        <v>16</v>
       </c>
       <c r="C28" t="n">
-        <v>103120</v>
+        <v>1992</v>
       </c>
       <c r="D28" t="n">
-        <v>41328</v>
+        <v>840</v>
       </c>
       <c r="E28" t="n">
-        <v>59.92</v>
+        <v>57.83</v>
       </c>
       <c r="F28" t="n">
-        <v>37752</v>
+        <v>840</v>
       </c>
       <c r="G28" t="n">
-        <v>63.39</v>
+        <v>57.83</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>f_100_200-1</t>
+          <t>sao2f1_100</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C29" t="n">
-        <v>102992</v>
+        <v>480</v>
       </c>
       <c r="D29" t="n">
-        <v>40616</v>
+        <v>480</v>
       </c>
       <c r="E29" t="n">
-        <v>60.56</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>30432</v>
+        <v>208</v>
       </c>
       <c r="G29" t="n">
-        <v>70.45</v>
+        <v>56.67</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>f_100_200-2</t>
+          <t>sao2f2_100</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C30" t="n">
-        <v>103336</v>
+        <v>608</v>
       </c>
       <c r="D30" t="n">
-        <v>40544</v>
+        <v>608</v>
       </c>
       <c r="E30" t="n">
-        <v>60.76</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>30152</v>
+        <v>240</v>
       </c>
       <c r="G30" t="n">
-        <v>70.81999999999999</v>
+        <v>60.53</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>f_100_200-3</t>
+          <t>sao2f3_100</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C31" t="n">
-        <v>102728</v>
+        <v>568</v>
       </c>
       <c r="D31" t="n">
-        <v>40640</v>
+        <v>392</v>
       </c>
       <c r="E31" t="n">
-        <v>60.44</v>
+        <v>30.99</v>
       </c>
       <c r="F31" t="n">
-        <v>36976</v>
+        <v>272</v>
       </c>
       <c r="G31" t="n">
-        <v>64.01000000000001</v>
+        <v>52.11</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>f_100_200-4</t>
+          <t>sao2f4_100</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C32" t="n">
-        <v>103304</v>
+        <v>536</v>
       </c>
       <c r="D32" t="n">
-        <v>40360</v>
+        <v>408</v>
       </c>
       <c r="E32" t="n">
-        <v>60.93</v>
+        <v>23.88</v>
       </c>
       <c r="F32" t="n">
-        <v>36848</v>
+        <v>280</v>
       </c>
       <c r="G32" t="n">
-        <v>64.33</v>
+        <v>47.76</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>f_100_400-0</t>
+          <t>sf_232</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="C33" t="n">
-        <v>206552</v>
+        <v>16</v>
       </c>
       <c r="D33" t="n">
-        <v>81264</v>
+        <v>8</v>
       </c>
       <c r="E33" t="n">
-        <v>60.66</v>
+        <v>50</v>
       </c>
       <c r="F33" t="n">
-        <v>68568</v>
+        <v>8</v>
       </c>
       <c r="G33" t="n">
-        <v>66.8</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>f_100_400-1</t>
+          <t>sym10_d_100</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C34" t="n">
-        <v>208152</v>
+        <v>3880</v>
       </c>
       <c r="D34" t="n">
-        <v>83392</v>
+        <v>3216</v>
       </c>
       <c r="E34" t="n">
-        <v>59.94</v>
+        <v>17.11</v>
       </c>
       <c r="F34" t="n">
-        <v>68600</v>
+        <v>1552</v>
       </c>
       <c r="G34" t="n">
-        <v>67.04000000000001</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>f_100_400-2</t>
+          <t>f_100_200-0</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>100</v>
       </c>
       <c r="C35" t="n">
-        <v>207768</v>
+        <v>103120</v>
       </c>
       <c r="D35" t="n">
-        <v>82640</v>
+        <v>41328</v>
       </c>
       <c r="E35" t="n">
-        <v>60.22</v>
+        <v>59.92</v>
       </c>
       <c r="F35" t="n">
-        <v>69896</v>
+        <v>37752</v>
       </c>
       <c r="G35" t="n">
-        <v>66.36</v>
+        <v>63.39</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>f_100_400-3</t>
+          <t>f_100_200-1</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>100</v>
       </c>
       <c r="C36" t="n">
-        <v>206600</v>
+        <v>102992</v>
       </c>
       <c r="D36" t="n">
-        <v>81840</v>
+        <v>40616</v>
       </c>
       <c r="E36" t="n">
-        <v>60.39</v>
+        <v>60.56</v>
       </c>
       <c r="F36" t="n">
-        <v>69176</v>
+        <v>30432</v>
       </c>
       <c r="G36" t="n">
-        <v>66.52</v>
+        <v>70.45</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>f_100_600-0</t>
+          <t>f_100_200-2</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>100</v>
       </c>
       <c r="C37" t="n">
-        <v>309384</v>
+        <v>103336</v>
       </c>
       <c r="D37" t="n">
-        <v>121312</v>
+        <v>40544</v>
       </c>
       <c r="E37" t="n">
-        <v>60.79</v>
+        <v>60.76</v>
       </c>
       <c r="F37" t="n">
-        <v>106272</v>
+        <v>30152</v>
       </c>
       <c r="G37" t="n">
-        <v>65.65000000000001</v>
+        <v>70.81999999999999</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>f_100_600-1</t>
+          <t>f_100_200-3</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>100</v>
       </c>
       <c r="C38" t="n">
-        <v>309648</v>
+        <v>102728</v>
       </c>
       <c r="D38" t="n">
-        <v>119976</v>
+        <v>40640</v>
       </c>
       <c r="E38" t="n">
-        <v>61.25</v>
+        <v>60.44</v>
       </c>
       <c r="F38" t="n">
-        <v>105576</v>
+        <v>36976</v>
       </c>
       <c r="G38" t="n">
-        <v>65.90000000000001</v>
+        <v>64.01000000000001</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>f_100_600-2</t>
+          <t>f_100_200-4</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>100</v>
       </c>
       <c r="C39" t="n">
-        <v>309744</v>
+        <v>103304</v>
       </c>
       <c r="D39" t="n">
-        <v>122984</v>
+        <v>40360</v>
       </c>
       <c r="E39" t="n">
-        <v>60.29</v>
+        <v>60.93</v>
       </c>
       <c r="F39" t="n">
-        <v>107440</v>
+        <v>36848</v>
       </c>
       <c r="G39" t="n">
-        <v>65.31</v>
+        <v>64.33</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>f_100_600-3</t>
+          <t>f_100_400-0</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>100</v>
       </c>
       <c r="C40" t="n">
-        <v>310400</v>
+        <v>206552</v>
       </c>
       <c r="D40" t="n">
-        <v>122336</v>
+        <v>81264</v>
       </c>
       <c r="E40" t="n">
-        <v>60.59</v>
+        <v>60.66</v>
       </c>
       <c r="F40" t="n">
-        <v>107680</v>
+        <v>68568</v>
       </c>
       <c r="G40" t="n">
-        <v>65.31</v>
+        <v>66.8</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>f_100_600-4</t>
+          <t>f_100_400-1</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>100</v>
       </c>
       <c r="C41" t="n">
-        <v>310392</v>
+        <v>208152</v>
       </c>
       <c r="D41" t="n">
-        <v>122000</v>
+        <v>83392</v>
       </c>
       <c r="E41" t="n">
-        <v>60.69</v>
+        <v>59.94</v>
       </c>
       <c r="F41" t="n">
-        <v>107168</v>
+        <v>68600</v>
       </c>
       <c r="G41" t="n">
-        <v>65.47</v>
+        <v>67.04000000000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>t481_d_100</t>
+          <t>f_100_400-2</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="C42" t="n">
-        <v>128</v>
+        <v>207768</v>
       </c>
       <c r="D42" t="n">
-        <v>64</v>
+        <v>82640</v>
       </c>
       <c r="E42" t="n">
-        <v>50</v>
+        <v>60.22</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>69896</v>
       </c>
       <c r="G42" t="n">
-        <v>100</v>
+        <v>66.36</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>xor5_d_100</t>
+          <t>f_100_400-3</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>206600</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>81840</v>
       </c>
       <c r="E43" t="n">
-        <v>0</v>
+        <v>60.39</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>69176</v>
       </c>
       <c r="G43" t="n">
-        <v>0</v>
+        <v>66.52</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>xor8</t>
+          <t>f_100_600-0</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="C44" t="n">
-        <v>40</v>
+        <v>309384</v>
       </c>
       <c r="D44" t="n">
-        <v>32</v>
+        <v>121312</v>
       </c>
       <c r="E44" t="n">
-        <v>20</v>
+        <v>60.79</v>
       </c>
       <c r="F44" t="n">
-        <v>32</v>
+        <v>106272</v>
       </c>
       <c r="G44" t="n">
-        <v>20</v>
+        <v>65.65000000000001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>f_100_600-1</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>100</v>
+      </c>
+      <c r="C45" t="n">
+        <v>309648</v>
+      </c>
+      <c r="D45" t="n">
+        <v>119976</v>
+      </c>
+      <c r="E45" t="n">
+        <v>61.25</v>
+      </c>
+      <c r="F45" t="n">
+        <v>105576</v>
+      </c>
+      <c r="G45" t="n">
+        <v>65.90000000000001</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>f_100_600-2</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>100</v>
+      </c>
+      <c r="C46" t="n">
+        <v>309744</v>
+      </c>
+      <c r="D46" t="n">
+        <v>122984</v>
+      </c>
+      <c r="E46" t="n">
+        <v>60.29</v>
+      </c>
+      <c r="F46" t="n">
+        <v>107440</v>
+      </c>
+      <c r="G46" t="n">
+        <v>65.31</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>f_100_600-3</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>100</v>
+      </c>
+      <c r="C47" t="n">
+        <v>310400</v>
+      </c>
+      <c r="D47" t="n">
+        <v>122336</v>
+      </c>
+      <c r="E47" t="n">
+        <v>60.59</v>
+      </c>
+      <c r="F47" t="n">
+        <v>107680</v>
+      </c>
+      <c r="G47" t="n">
+        <v>65.31</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>f_100_600-4</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>100</v>
+      </c>
+      <c r="C48" t="n">
+        <v>310392</v>
+      </c>
+      <c r="D48" t="n">
+        <v>122000</v>
+      </c>
+      <c r="E48" t="n">
+        <v>60.69</v>
+      </c>
+      <c r="F48" t="n">
+        <v>107168</v>
+      </c>
+      <c r="G48" t="n">
+        <v>65.47</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>t481_d_100</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>16</v>
+      </c>
+      <c r="C49" t="n">
+        <v>128</v>
+      </c>
+      <c r="D49" t="n">
+        <v>64</v>
+      </c>
+      <c r="E49" t="n">
+        <v>50</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>xor5_d_100</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>5</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>xor8</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>8</v>
+      </c>
+      <c r="C51" t="n">
+        <v>40</v>
+      </c>
+      <c r="D51" t="n">
+        <v>32</v>
+      </c>
+      <c r="E51" t="n">
+        <v>20</v>
+      </c>
+      <c r="F51" t="n">
+        <v>32</v>
+      </c>
+      <c r="G51" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>z42</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B52" t="n">
         <v>7</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C52" t="n">
         <v>152</v>
       </c>
-      <c r="D45" t="n">
+      <c r="D52" t="n">
         <v>120</v>
       </c>
-      <c r="E45" t="n">
+      <c r="E52" t="n">
         <v>21.05</v>
       </c>
-      <c r="F45" t="n">
+      <c r="F52" t="n">
         <v>80</v>
       </c>
-      <c r="G45" t="n">
+      <c r="G52" t="n">
         <v>47.37</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixing the logic for synthetic functions. Regenerating results.
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maslov Cost" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T-Count" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structure" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Maslov Cost" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="T-Count" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resources" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Structure" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,37 +420,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ESOP Cost</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EOSOPS Cost</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>EOSOPS Cost Saving (%)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Final Cost</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Final Cost Saving (%)</t>
         </is>
@@ -637,10 +625,10 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G8" t="n">
-        <v>27.94</v>
+        <v>22.06</v>
       </c>
     </row>
     <row r="9">
@@ -737,10 +725,10 @@
         <v>32.62</v>
       </c>
       <c r="F12" t="n">
-        <v>4496</v>
+        <v>4305</v>
       </c>
       <c r="G12" t="n">
-        <v>65.7</v>
+        <v>67.16</v>
       </c>
     </row>
     <row r="13">
@@ -787,10 +775,10 @@
         <v>10.74</v>
       </c>
       <c r="F14" t="n">
-        <v>4711</v>
+        <v>4695</v>
       </c>
       <c r="G14" t="n">
-        <v>67.23</v>
+        <v>67.34999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -837,10 +825,10 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="G16" t="n">
-        <v>67.23</v>
+        <v>66.59</v>
       </c>
     </row>
     <row r="17">
@@ -1012,10 +1000,10 @@
         <v>1.12</v>
       </c>
       <c r="F23" t="n">
-        <v>531</v>
+        <v>511</v>
       </c>
       <c r="G23" t="n">
-        <v>60.4</v>
+        <v>61.89</v>
       </c>
     </row>
     <row r="24">
@@ -1112,10 +1100,10 @@
         <v>30.11</v>
       </c>
       <c r="F27" t="n">
-        <v>1662</v>
+        <v>1714</v>
       </c>
       <c r="G27" t="n">
-        <v>64.61</v>
+        <v>63.5</v>
       </c>
     </row>
     <row r="28">
@@ -1162,10 +1150,10 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>1823</v>
+        <v>1971</v>
       </c>
       <c r="G29" t="n">
-        <v>64.73999999999999</v>
+        <v>61.88</v>
       </c>
     </row>
     <row r="30">
@@ -1187,10 +1175,10 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>2466</v>
+        <v>2610</v>
       </c>
       <c r="G30" t="n">
-        <v>70.15000000000001</v>
+        <v>68.40000000000001</v>
       </c>
     </row>
     <row r="31">
@@ -1287,10 +1275,10 @@
         <v>24.27</v>
       </c>
       <c r="F34" t="n">
-        <v>16825</v>
+        <v>16573</v>
       </c>
       <c r="G34" t="n">
-        <v>67.14</v>
+        <v>67.63</v>
       </c>
     </row>
     <row r="35">
@@ -1306,16 +1294,16 @@
         <v>11983160</v>
       </c>
       <c r="D35" t="n">
-        <v>4063972</v>
+        <v>11983160</v>
       </c>
       <c r="E35" t="n">
-        <v>66.09</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>2696428</v>
+        <v>8143072</v>
       </c>
       <c r="G35" t="n">
-        <v>77.5</v>
+        <v>32.05</v>
       </c>
     </row>
     <row r="36">
@@ -1331,16 +1319,16 @@
         <v>11966928</v>
       </c>
       <c r="D36" t="n">
-        <v>3980238</v>
+        <v>11966928</v>
       </c>
       <c r="E36" t="n">
-        <v>66.73999999999999</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>2180060</v>
+        <v>8099976</v>
       </c>
       <c r="G36" t="n">
-        <v>81.78</v>
+        <v>32.31</v>
       </c>
     </row>
     <row r="37">
@@ -1356,16 +1344,16 @@
         <v>12010942</v>
       </c>
       <c r="D37" t="n">
-        <v>3969852</v>
+        <v>12010942</v>
       </c>
       <c r="E37" t="n">
-        <v>66.95</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>2159279</v>
+        <v>8155314</v>
       </c>
       <c r="G37" t="n">
-        <v>82.02</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="38">
@@ -1381,16 +1369,16 @@
         <v>11933054</v>
       </c>
       <c r="D38" t="n">
-        <v>3977013</v>
+        <v>11933054</v>
       </c>
       <c r="E38" t="n">
-        <v>66.67</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>2623863</v>
+        <v>8078358</v>
       </c>
       <c r="G38" t="n">
-        <v>78.01000000000001</v>
+        <v>32.3</v>
       </c>
     </row>
     <row r="39">
@@ -1406,16 +1394,16 @@
         <v>12006782</v>
       </c>
       <c r="D39" t="n">
-        <v>3940042</v>
+        <v>12006782</v>
       </c>
       <c r="E39" t="n">
-        <v>67.18000000000001</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>2594760</v>
+        <v>8124438</v>
       </c>
       <c r="G39" t="n">
-        <v>78.39</v>
+        <v>32.33</v>
       </c>
     </row>
     <row r="40">
@@ -1431,16 +1419,16 @@
         <v>24006252</v>
       </c>
       <c r="D40" t="n">
-        <v>7963508</v>
+        <v>24006252</v>
       </c>
       <c r="E40" t="n">
-        <v>66.83</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>4915732</v>
+        <v>16078700</v>
       </c>
       <c r="G40" t="n">
-        <v>79.52</v>
+        <v>33.02</v>
       </c>
     </row>
     <row r="41">
@@ -1456,16 +1444,16 @@
         <v>24211430</v>
       </c>
       <c r="D41" t="n">
-        <v>8226180</v>
+        <v>24211430</v>
       </c>
       <c r="E41" t="n">
-        <v>66.02</v>
+        <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>4938720</v>
+        <v>16259930</v>
       </c>
       <c r="G41" t="n">
-        <v>79.59999999999999</v>
+        <v>32.84</v>
       </c>
     </row>
     <row r="42">
@@ -1481,16 +1469,16 @@
         <v>24161902</v>
       </c>
       <c r="D42" t="n">
-        <v>8136935</v>
+        <v>24161902</v>
       </c>
       <c r="E42" t="n">
-        <v>66.31999999999999</v>
+        <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>5065613</v>
+        <v>16217954</v>
       </c>
       <c r="G42" t="n">
-        <v>79.03</v>
+        <v>32.88</v>
       </c>
     </row>
     <row r="43">
@@ -1506,16 +1494,16 @@
         <v>24012388</v>
       </c>
       <c r="D43" t="n">
-        <v>8038699</v>
+        <v>24012388</v>
       </c>
       <c r="E43" t="n">
-        <v>66.52</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>4993927</v>
+        <v>16142304</v>
       </c>
       <c r="G43" t="n">
-        <v>79.2</v>
+        <v>32.78</v>
       </c>
     </row>
     <row r="44">
@@ -1531,16 +1519,16 @@
         <v>35952736</v>
       </c>
       <c r="D44" t="n">
-        <v>11877928</v>
+        <v>35952736</v>
       </c>
       <c r="E44" t="n">
-        <v>66.95999999999999</v>
+        <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>7642677</v>
+        <v>23967252</v>
       </c>
       <c r="G44" t="n">
-        <v>78.73999999999999</v>
+        <v>33.34</v>
       </c>
     </row>
     <row r="45">
@@ -1556,16 +1544,16 @@
         <v>35986554</v>
       </c>
       <c r="D45" t="n">
-        <v>11703342</v>
+        <v>35986554</v>
       </c>
       <c r="E45" t="n">
-        <v>67.48</v>
+        <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>7566845</v>
+        <v>23984750</v>
       </c>
       <c r="G45" t="n">
-        <v>78.97</v>
+        <v>33.35</v>
       </c>
     </row>
     <row r="46">
@@ -1581,16 +1569,16 @@
         <v>35999290</v>
       </c>
       <c r="D46" t="n">
-        <v>12085226</v>
+        <v>35999290</v>
       </c>
       <c r="E46" t="n">
-        <v>66.43000000000001</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>7741225</v>
+        <v>24033046</v>
       </c>
       <c r="G46" t="n">
-        <v>78.5</v>
+        <v>33.24</v>
       </c>
     </row>
     <row r="47">
@@ -1606,16 +1594,16 @@
         <v>36082960</v>
       </c>
       <c r="D47" t="n">
-        <v>11999517</v>
+        <v>36082960</v>
       </c>
       <c r="E47" t="n">
-        <v>66.73999999999999</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>7786433</v>
+        <v>24030852</v>
       </c>
       <c r="G47" t="n">
-        <v>78.42</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="48">
@@ -1631,16 +1619,16 @@
         <v>36081916</v>
       </c>
       <c r="D48" t="n">
-        <v>11961918</v>
+        <v>36081916</v>
       </c>
       <c r="E48" t="n">
-        <v>66.84999999999999</v>
+        <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>7729276</v>
+        <v>24041996</v>
       </c>
       <c r="G48" t="n">
-        <v>78.58</v>
+        <v>33.37</v>
       </c>
     </row>
     <row r="49">
@@ -1733,37 +1721,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ESOP T</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EOSOPS T</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>EOSOPS T Saving (%)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Final T</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Final T Saving (%)</t>
         </is>
@@ -2048,10 +2036,10 @@
         <v>19.05</v>
       </c>
       <c r="F12" t="n">
-        <v>656</v>
+        <v>644</v>
       </c>
       <c r="G12" t="n">
-        <v>39.93</v>
+        <v>41.03</v>
       </c>
     </row>
     <row r="13">
@@ -2503,10 +2491,10 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="G29" t="n">
-        <v>42.86</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30">
@@ -2528,10 +2516,10 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="G30" t="n">
-        <v>43.18</v>
+        <v>45.45</v>
       </c>
     </row>
     <row r="31">
@@ -2628,10 +2616,10 @@
         <v>12.35</v>
       </c>
       <c r="F34" t="n">
-        <v>1284</v>
+        <v>1296</v>
       </c>
       <c r="G34" t="n">
-        <v>43.39</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="35">
@@ -2647,16 +2635,16 @@
         <v>52360</v>
       </c>
       <c r="D35" t="n">
-        <v>21472</v>
+        <v>52360</v>
       </c>
       <c r="E35" t="n">
-        <v>58.99</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>21252</v>
+        <v>40184</v>
       </c>
       <c r="G35" t="n">
-        <v>59.41</v>
+        <v>23.25</v>
       </c>
     </row>
     <row r="36">
@@ -2672,16 +2660,16 @@
         <v>52296</v>
       </c>
       <c r="D36" t="n">
-        <v>21132</v>
+        <v>52296</v>
       </c>
       <c r="E36" t="n">
-        <v>59.59</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>17088</v>
+        <v>40016</v>
       </c>
       <c r="G36" t="n">
-        <v>67.31999999999999</v>
+        <v>23.48</v>
       </c>
     </row>
     <row r="37">
@@ -2697,16 +2685,16 @@
         <v>52468</v>
       </c>
       <c r="D37" t="n">
-        <v>21096</v>
+        <v>52468</v>
       </c>
       <c r="E37" t="n">
-        <v>59.79</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>16964</v>
+        <v>40232</v>
       </c>
       <c r="G37" t="n">
-        <v>67.67</v>
+        <v>23.32</v>
       </c>
     </row>
     <row r="38">
@@ -2722,16 +2710,16 @@
         <v>52164</v>
       </c>
       <c r="D38" t="n">
-        <v>21132</v>
+        <v>52164</v>
       </c>
       <c r="E38" t="n">
-        <v>59.49</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>20852</v>
+        <v>39932</v>
       </c>
       <c r="G38" t="n">
-        <v>60.03</v>
+        <v>23.45</v>
       </c>
     </row>
     <row r="39">
@@ -2747,16 +2735,16 @@
         <v>52452</v>
       </c>
       <c r="D39" t="n">
-        <v>20988</v>
+        <v>52452</v>
       </c>
       <c r="E39" t="n">
-        <v>59.99</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>20784</v>
+        <v>40112</v>
       </c>
       <c r="G39" t="n">
-        <v>60.38</v>
+        <v>23.53</v>
       </c>
     </row>
     <row r="40">
@@ -2772,16 +2760,16 @@
         <v>104876</v>
       </c>
       <c r="D40" t="n">
-        <v>42288</v>
+        <v>104876</v>
       </c>
       <c r="E40" t="n">
-        <v>59.68</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>38536</v>
+        <v>79560</v>
       </c>
       <c r="G40" t="n">
-        <v>63.26</v>
+        <v>24.14</v>
       </c>
     </row>
     <row r="41">
@@ -2797,16 +2785,16 @@
         <v>105676</v>
       </c>
       <c r="D41" t="n">
-        <v>43328</v>
+        <v>105676</v>
       </c>
       <c r="E41" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>38540</v>
+        <v>80268</v>
       </c>
       <c r="G41" t="n">
-        <v>63.53</v>
+        <v>24.04</v>
       </c>
     </row>
     <row r="42">
@@ -2822,16 +2810,16 @@
         <v>105484</v>
       </c>
       <c r="D42" t="n">
-        <v>42980</v>
+        <v>105484</v>
       </c>
       <c r="E42" t="n">
-        <v>59.25</v>
+        <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>39216</v>
+        <v>80104</v>
       </c>
       <c r="G42" t="n">
-        <v>62.82</v>
+        <v>24.06</v>
       </c>
     </row>
     <row r="43">
@@ -2847,16 +2835,16 @@
         <v>104900</v>
       </c>
       <c r="D43" t="n">
-        <v>42556</v>
+        <v>104900</v>
       </c>
       <c r="E43" t="n">
-        <v>59.43</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>38836</v>
+        <v>79808</v>
       </c>
       <c r="G43" t="n">
-        <v>62.98</v>
+        <v>23.92</v>
       </c>
     </row>
     <row r="44">
@@ -2872,16 +2860,16 @@
         <v>157092</v>
       </c>
       <c r="D44" t="n">
-        <v>63176</v>
+        <v>157092</v>
       </c>
       <c r="E44" t="n">
-        <v>59.78</v>
+        <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>59784</v>
+        <v>118752</v>
       </c>
       <c r="G44" t="n">
-        <v>61.94</v>
+        <v>24.41</v>
       </c>
     </row>
     <row r="45">
@@ -2897,16 +2885,16 @@
         <v>157224</v>
       </c>
       <c r="D45" t="n">
-        <v>62500</v>
+        <v>157224</v>
       </c>
       <c r="E45" t="n">
-        <v>60.25</v>
+        <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>59436</v>
+        <v>118820</v>
       </c>
       <c r="G45" t="n">
-        <v>62.2</v>
+        <v>24.43</v>
       </c>
     </row>
     <row r="46">
@@ -2922,16 +2910,16 @@
         <v>157272</v>
       </c>
       <c r="D46" t="n">
-        <v>63980</v>
+        <v>157272</v>
       </c>
       <c r="E46" t="n">
-        <v>59.32</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>60356</v>
+        <v>119008</v>
       </c>
       <c r="G46" t="n">
-        <v>61.62</v>
+        <v>24.33</v>
       </c>
     </row>
     <row r="47">
@@ -2947,16 +2935,16 @@
         <v>157600</v>
       </c>
       <c r="D47" t="n">
-        <v>63660</v>
+        <v>157600</v>
       </c>
       <c r="E47" t="n">
-        <v>59.61</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>60488</v>
+        <v>119000</v>
       </c>
       <c r="G47" t="n">
-        <v>61.62</v>
+        <v>24.49</v>
       </c>
     </row>
     <row r="48">
@@ -2972,16 +2960,16 @@
         <v>157596</v>
       </c>
       <c r="D48" t="n">
-        <v>63512</v>
+        <v>157596</v>
       </c>
       <c r="E48" t="n">
-        <v>59.7</v>
+        <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>60240</v>
+        <v>119044</v>
       </c>
       <c r="G48" t="n">
-        <v>61.78</v>
+        <v>24.46</v>
       </c>
     </row>
     <row r="49">
@@ -3084,52 +3072,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ESOP Gates</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Final Gates</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>ESOP Max Controls</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Final Max Controls</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Ancilla Peak</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Ancilla Total</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ESOP Histogram</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Final Histogram</t>
         </is>
@@ -3382,7 +3370,7 @@
         <v>4</v>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
@@ -3397,7 +3385,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1:1 2:2 3:2</t>
+          <t>1:1 2:3 4:1</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3516,7 @@
         <v>50</v>
       </c>
       <c r="D12" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E12" t="n">
         <v>9</v>
@@ -3540,7 +3528,7 @@
         <v>2</v>
       </c>
       <c r="H12" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -3549,7 +3537,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1:9 2:21 3:6 4:1 5:7 6:10 7:6 8:2</t>
+          <t>1:10 2:20 3:7 4:3 5:7 6:8 7:6 8:2</t>
         </is>
       </c>
     </row>
@@ -3625,7 +3613,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>1:13 2:18 3:5 4:2 5:2 6:8 7:9 8:2</t>
+          <t>1:13 2:18 3:4 4:4 5:1 6:8 7:9 8:2</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3689,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>1:3 2:1 3:3 4:1 5:1 7:1</t>
+          <t>1:4 3:2 4:2 5:1 7:1</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3955,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>1:7 2:11 3:3 4:5 5:4</t>
+          <t>1:6 2:12 3:3 4:6 5:3</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4107,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>1:15 2:11 3:3 4:1 5:12 6:4 7:1</t>
+          <t>1:16 2:10 3:3 4:1 5:11 6:5 7:1</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4183,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>1:6 3:2 4:2 5:1 6:1 8:3</t>
+          <t>1:6 3:3 6:3 8:3</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4221,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>1:4 2:6 4:2 5:1 7:1 8:4</t>
+          <t>1:4 2:8 7:2 8:4</t>
         </is>
       </c>
     </row>
@@ -4385,7 +4373,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>1:24 2:36 3:6 4:2 6:5 7:22 8:10 9:5</t>
+          <t>1:23 2:33 3:9 4:3 5:1 6:6 7:20 8:10 9:5</t>
         </is>
       </c>
     </row>
@@ -4402,28 +4390,28 @@
         <v>200</v>
       </c>
       <c r="D35" t="n">
-        <v>396</v>
+        <v>300</v>
       </c>
       <c r="E35" t="n">
         <v>78</v>
       </c>
       <c r="F35" t="n">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H35" t="n">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>53:1 54:1 55:1 56:1 57:2 58:3 59:4 60:8 61:9 62:14 63:11</t>
+          <t>53:1 54:1 55:1 56:1 57:2 58:3 59:4 60:8 61:9 62:14 63:11 64:9 65:23 66:12 67:14 68:14 69:14 70:19 71:13 72:11 73:4 74:5 75:3 76:2 77:1 78:1</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>4:6 5:5 6:10 7:18 8:19 9:35 10:28 11:33 12:27 13:24 14:20 15:29 16:7 17:20 18:6 19:19 20:11 21:25 22:4 23:18 24:3 25:12 26:2 27:7 28:4 29:2 31:2</t>
+          <t>16:1 19:1 20:2 22:1 24:1 25:1 26:5 27:5 28:6 29:12 30:10 31:15 32:22 33:28 34:27 35:32 36:36 37:24 38:25 39:20 40:9 41:9 42:1 43:6 45:1</t>
         </is>
       </c>
     </row>
@@ -4440,28 +4428,28 @@
         <v>200</v>
       </c>
       <c r="D36" t="n">
-        <v>338</v>
+        <v>300</v>
       </c>
       <c r="E36" t="n">
         <v>79</v>
       </c>
       <c r="F36" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="G36" t="n">
         <v>2</v>
       </c>
       <c r="H36" t="n">
-        <v>168</v>
+        <v>200</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>53:1 55:2 56:2 57:2 58:3 59:5 60:7 61:7 62:9 63:14</t>
+          <t>53:1 55:2 56:2 57:2 58:3 59:5 60:7 61:7 62:9 63:14 64:11 65:24 66:17 67:21 68:12 69:10 70:17 71:11 72:8 73:3 74:5 75:2 76:1 77:2 78:2 79:2</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>0:14 1:9 2:1 3:1 4:1 5:1 6:6 7:16 8:23 9:18 10:28 11:19 12:21 13:17 14:18 15:21 16:16 17:18 18:12 19:16 20:7 21:14 22:5 23:12 24:5 25:4 26:4 27:3 28:3 29:2 30:1 35:1 36:1</t>
+          <t>16:1 21:1 22:3 25:4 26:3 27:5 28:5 29:13 30:10 31:15 32:20 33:24 34:45 35:37 36:28 37:29 38:15 39:15 40:11 41:8 42:6 45:1 48:1</t>
         </is>
       </c>
     </row>
@@ -4478,28 +4466,28 @@
         <v>200</v>
       </c>
       <c r="D37" t="n">
-        <v>355</v>
+        <v>300</v>
       </c>
       <c r="E37" t="n">
         <v>81</v>
       </c>
       <c r="F37" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="G37" t="n">
         <v>2</v>
       </c>
       <c r="H37" t="n">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>53:1 54:1 56:1 58:5 59:2 60:7 61:9 62:20 63:13</t>
+          <t>53:1 54:1 56:1 58:5 59:2 60:7 61:9 62:20 63:13 64:16 65:16 66:11 67:15 68:11 69:14 70:14 71:9 72:11 73:9 74:4 75:3 76:3 77:2 78:1 79:1 81:1</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>0:24 1:15 2:2 4:2 5:3 6:14 7:8 8:22 9:22 10:24 11:23 12:23 13:21 14:13 15:16 16:10 17:20 18:8 19:18 20:6 21:20 22:5 23:11 24:9 25:1 26:1 27:8 28:1 29:3 30:1 35:1</t>
+          <t>19:1 21:1 22:1 23:2 24:2 25:2 26:6 27:4 28:2 29:15 30:9 31:16 32:23 33:22 34:28 35:29 36:32 37:32 38:26 39:22 40:15 41:5 42:2 43:1 44:2</t>
         </is>
       </c>
     </row>
@@ -4516,28 +4504,28 @@
         <v>200</v>
       </c>
       <c r="D38" t="n">
-        <v>394</v>
+        <v>300</v>
       </c>
       <c r="E38" t="n">
         <v>78</v>
       </c>
       <c r="F38" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H38" t="n">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>52:1 55:2 56:1 57:2 58:3 59:11 60:4 61:8 62:8 63:16</t>
+          <t>52:1 55:2 56:1 57:2 58:3 59:11 60:4 61:8 62:8 63:16 64:7 65:21 66:24 67:18 68:13 69:11 70:13 71:9 72:8 73:8 74:8 75:1 77:2 78:1</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>3:2 4:4 5:9 6:11 7:17 8:19 9:30 10:33 11:30 12:24 13:33 14:14 15:24 16:12 17:21 18:8 19:20 20:11 21:17 22:8 23:16 24:7 25:9 26:5 27:5 29:3 30:1 31:1</t>
+          <t>17:1 20:1 23:1 24:5 25:3 26:3 27:6 28:4 29:9 30:13 31:21 32:18 33:30 34:20 35:46 36:35 37:20 38:23 39:16 40:14 41:6 42:1 43:4</t>
         </is>
       </c>
     </row>
@@ -4554,28 +4542,28 @@
         <v>200</v>
       </c>
       <c r="D39" t="n">
-        <v>394</v>
+        <v>300</v>
       </c>
       <c r="E39" t="n">
         <v>78</v>
       </c>
       <c r="F39" t="n">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H39" t="n">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>54:1 56:4 57:2 58:1 59:4 60:5 61:9 62:10 63:16</t>
+          <t>54:1 56:4 57:2 58:1 59:4 60:5 61:9 62:10 63:16 64:9 65:16 66:18 67:16 68:22 69:18 70:11 71:12 72:8 73:8 74:1 75:6 76:2 78:1</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>3:1 4:2 5:4 6:9 7:32 8:24 9:26 10:29 11:26 12:17 13:38 14:16 15:30 16:14 17:21 18:9 19:23 20:5 21:19 22:7 23:12 24:6 25:7 26:2 27:7 28:2 29:4 31:1 35:1</t>
+          <t>14:1 21:1 22:2 23:1 24:1 25:4 26:4 27:5 28:7 29:6 30:13 31:18 32:14 33:29 34:31 35:31 36:36 37:27 38:27 39:20 40:13 41:4 42:2 43:2 46:1</t>
         </is>
       </c>
     </row>
@@ -4592,28 +4580,28 @@
         <v>400</v>
       </c>
       <c r="D40" t="n">
-        <v>783</v>
+        <v>600</v>
       </c>
       <c r="E40" t="n">
         <v>81</v>
       </c>
       <c r="F40" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="G40" t="n">
         <v>2</v>
       </c>
       <c r="H40" t="n">
-        <v>389</v>
+        <v>400</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>52:2 55:1 56:1 57:5 58:5 59:19 60:15 61:12 62:23 63:25</t>
+          <t>52:2 55:1 56:1 57:5 58:5 59:19 60:15 61:12 62:23 63:25 64:33 65:23 66:24 67:33 68:39 69:25 70:21 71:40 72:14 73:19 74:8 75:3 76:5 77:2 78:1 81:2</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>0:43 1:28 2:4 4:1 5:10 6:17 7:30 8:38 9:56 10:49 11:58 12:42 13:50 14:40 15:45 16:27 17:36 18:16 19:44 20:14 21:35 22:17 23:26 24:14 25:14 26:4 27:14 28:4 29:2 30:2 31:2 32:1</t>
+          <t>14:1 19:1 21:1 22:2 24:2 25:5 26:10 27:11 28:10 29:11 30:36 31:38 32:50 33:64 34:51 35:76 36:69 37:50 38:58 39:30 40:12 41:5 42:3 44:2 45:1 47:1</t>
         </is>
       </c>
     </row>
@@ -4630,28 +4618,28 @@
         <v>400</v>
       </c>
       <c r="D41" t="n">
-        <v>749</v>
+        <v>600</v>
       </c>
       <c r="E41" t="n">
         <v>82</v>
       </c>
       <c r="F41" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="G41" t="n">
         <v>2</v>
       </c>
       <c r="H41" t="n">
-        <v>373</v>
+        <v>400</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>52:1 53:1 55:2 56:2 57:2 58:4 59:16 60:10 61:22 62:16 63:21</t>
+          <t>52:1 53:1 55:2 56:2 57:2 58:4 59:16 60:10 61:22 62:16 63:21 64:24 65:28 66:32 67:33 68:42 69:31 70:30 71:11 72:8 73:15 74:12 75:12 76:11 77:5 78:4 79:4 82:1</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>0:23 1:16 2:2 3:1 4:2 5:14 6:19 7:20 8:51 9:59 10:49 11:47 12:40 13:52 14:31 15:37 16:24 17:57 18:18 19:40 20:21 21:32 22:8 23:21 24:14 25:15 26:12 27:5 28:4 29:6 30:4 31:3 33:1 37:1</t>
+          <t>16:1 20:1 23:2 24:6 25:6 26:4 27:11 28:13 29:14 30:23 31:28 32:49 33:52 34:63 35:78 36:71 37:58 38:45 39:35 40:22 41:12 42:3 43:2 45:1</t>
         </is>
       </c>
     </row>
@@ -4668,28 +4656,28 @@
         <v>400</v>
       </c>
       <c r="D42" t="n">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="E42" t="n">
         <v>79</v>
       </c>
       <c r="F42" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="G42" t="n">
         <v>2</v>
       </c>
       <c r="H42" t="n">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>54:2 55:1 56:4 57:1 58:7 59:10 60:9 61:23 62:16 63:14</t>
+          <t>54:2 55:1 56:4 57:1 58:7 59:10 60:9 61:23 62:16 63:14 64:36 65:32 66:32 67:30 68:29 69:34 70:23 71:25 72:24 73:18 74:11 75:8 76:4 77:2 78:4 79:1</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>0:53 1:34 2:5 5:1 6:23 7:25 8:43 9:48 10:59 11:52 12:42 13:52 14:35 15:35 16:26 17:48 18:20 19:42 20:17 21:44 22:13 23:23 24:12 25:18 26:6 27:9 28:3 29:2 30:6 31:1 32:2 33:1</t>
+          <t>15:1 19:2 21:1 22:1 23:2 24:1 25:4 26:1 27:6 28:17 29:22 30:23 31:32 32:45 33:50 34:76 35:76 36:64 37:61 38:51 39:32 40:21 41:8 42:2 43:1</t>
         </is>
       </c>
     </row>
@@ -4706,28 +4694,28 @@
         <v>400</v>
       </c>
       <c r="D43" t="n">
-        <v>766</v>
+        <v>600</v>
       </c>
       <c r="E43" t="n">
         <v>78</v>
       </c>
       <c r="F43" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="G43" t="n">
         <v>2</v>
       </c>
       <c r="H43" t="n">
-        <v>381</v>
+        <v>400</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>52:1 53:1 55:2 56:2 57:3 58:5 59:7 60:9 61:18 62:22 63:24</t>
+          <t>52:1 53:1 55:2 56:2 57:3 58:5 59:7 60:9 61:18 62:22 63:24 64:33 65:38 66:43 67:26 68:36 69:31 70:19 71:20 72:18 73:21 74:8 75:4 76:6 78:3</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>0:33 1:22 2:3 4:5 5:3 6:21 7:25 8:45 9:54 10:49 11:47 12:42 13:54 14:32 15:48 16:22 17:47 18:19 19:35 20:22 21:42 22:15 23:25 24:14 25:16 26:7 27:5 28:1 29:8 30:2 31:3</t>
+          <t>12:1 18:1 21:1 22:3 23:1 24:3 25:3 26:3 27:9 28:8 29:20 30:23 31:45 32:51 33:44 34:80 35:69 36:70 37:59 38:49 39:33 40:12 41:9 42:1 45:1 48:1</t>
         </is>
       </c>
     </row>
@@ -4744,28 +4732,28 @@
         <v>600</v>
       </c>
       <c r="D44" t="n">
-        <v>1278</v>
+        <v>900</v>
       </c>
       <c r="E44" t="n">
         <v>82</v>
       </c>
       <c r="F44" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="G44" t="n">
         <v>2</v>
       </c>
       <c r="H44" t="n">
-        <v>633</v>
+        <v>600</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>51:1 55:4 56:4 57:11 58:12 59:12 60:21 61:27 62:35 63:43</t>
+          <t>51:1 55:4 56:4 57:11 58:12 59:12 60:21 61:27 62:35 63:43 64:46 65:47 66:41 67:44 68:43 69:45 70:40 71:31 72:33 73:14 74:16 75:11 76:7 77:4 78:4 79:3 82:1</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>0:100 1:66 2:12 3:1 4:5 5:13 6:35 7:49 8:60 9:70 10:85 11:94 12:61 13:88 14:42 15:69 16:36 17:64 18:21 19:66 20:26 21:63 22:19 23:45 24:23 25:27 26:6 27:5 28:11 29:10 30:1 32:3 33:2</t>
+          <t>17:1 20:1 21:1 23:6 24:3 25:2 26:11 27:18 28:13 29:26 30:41 31:66 32:85 33:87 34:127 35:108 36:103 37:74 38:43 39:49 40:21 41:7 42:4 43:3</t>
         </is>
       </c>
     </row>
@@ -4782,28 +4770,28 @@
         <v>600</v>
       </c>
       <c r="D45" t="n">
-        <v>1245</v>
+        <v>900</v>
       </c>
       <c r="E45" t="n">
         <v>81</v>
       </c>
       <c r="F45" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="G45" t="n">
         <v>2</v>
       </c>
       <c r="H45" t="n">
-        <v>618</v>
+        <v>600</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>52:1 53:1 54:3 55:5 56:6 57:16 58:8 59:14 60:17 61:23 62:31 63:36</t>
+          <t>52:1 53:1 54:3 55:5 56:6 57:16 58:8 59:14 60:17 61:23 62:31 63:36 64:41 65:48 66:44 67:52 68:39 69:48 70:43 71:29 72:17 73:36 74:11 75:7 76:6 77:10 78:3 79:4 81:1</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>0:81 1:53 2:9 3:1 4:4 5:15 6:47 7:45 8:63 9:78 10:93 11:75 12:62 13:91 14:34 15:70 16:34 17:66 18:30 19:66 20:23 21:52 22:14 23:48 24:18 25:24 26:15 27:8 28:1 29:10 30:7 31:4 32:3 37:1</t>
+          <t>18:1 19:1 20:1 21:1 22:2 23:3 24:4 25:6 26:12 27:13 28:26 29:31 30:38 31:46 32:76 33:110 34:104 35:101 36:99 37:82 38:63 39:37 40:25 41:13 42:4 43:1</t>
         </is>
       </c>
     </row>
@@ -4820,28 +4808,28 @@
         <v>600</v>
       </c>
       <c r="D46" t="n">
-        <v>1211</v>
+        <v>900</v>
       </c>
       <c r="E46" t="n">
         <v>86</v>
       </c>
       <c r="F46" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="G46" t="n">
         <v>2</v>
       </c>
       <c r="H46" t="n">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>51:1 52:1 53:2 54:2 56:6 57:12 58:11 59:13 60:21 61:18 62:31 63:35</t>
+          <t>51:1 52:1 53:2 54:2 56:6 57:12 58:11 59:13 60:21 61:18 62:31 63:35 64:42 65:47 66:54 67:51 68:47 69:37 70:36 71:42 72:31 73:22 74:13 75:11 76:6 77:1 78:4 80:2 86:1</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>0:63 1:40 2:6 3:1 4:5 5:8 6:24 7:45 8:70 9:80 10:83 11:76 12:76 13:83 14:44 15:74 16:28 17:66 18:36 19:74 20:27 21:49 22:19 23:43 24:20 25:25 26:8 27:18 28:3 29:8 30:3 31:2 32:2 34:1 35:1</t>
+          <t>10:1 18:1 21:2 22:3 23:4 24:3 25:5 26:10 27:11 28:12 29:37 30:39 31:50 32:76 33:87 34:112 35:125 36:104 37:97 38:52 39:40 40:18 41:4 42:3 43:2 45:2</t>
         </is>
       </c>
     </row>
@@ -4858,28 +4846,28 @@
         <v>600</v>
       </c>
       <c r="D47" t="n">
-        <v>1245</v>
+        <v>900</v>
       </c>
       <c r="E47" t="n">
         <v>79</v>
       </c>
       <c r="F47" t="n">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="G47" t="n">
         <v>2</v>
       </c>
       <c r="H47" t="n">
-        <v>618</v>
+        <v>600</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>52:2 53:1 54:2 55:1 56:3 57:3 58:9 59:15 60:12 61:31 62:33 63:36</t>
+          <t>52:2 53:1 54:2 55:1 56:3 57:3 58:9 59:15 60:12 61:31 62:33 63:36 64:48 65:39 66:50 67:49 68:52 69:52 70:47 71:31 72:26 73:16 74:14 75:13 76:7 77:4 78:3 79:1</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>0:82 1:52 2:9 4:5 5:9 6:27 7:60 8:52 9:76 10:79 11:88 12:73 13:84 14:43 15:75 16:34 17:61 18:23 19:68 20:33 21:56 22:17 23:44 24:20 25:27 26:12 27:15 28:6 29:4 30:3 31:1 32:3 33:3 34:1</t>
+          <t>16:1 20:2 21:1 22:2 23:1 24:4 25:3 26:9 27:14 28:18 29:25 30:41 31:42 32:94 33:98 34:113 35:112 36:118 37:82 38:53 39:37 40:17 41:9 42:2 43:2</t>
         </is>
       </c>
     </row>
@@ -4896,28 +4884,28 @@
         <v>600</v>
       </c>
       <c r="D48" t="n">
-        <v>1262</v>
+        <v>900</v>
       </c>
       <c r="E48" t="n">
         <v>85</v>
       </c>
       <c r="F48" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="G48" t="n">
         <v>2</v>
       </c>
       <c r="H48" t="n">
-        <v>626</v>
+        <v>600</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>54:3 55:4 56:4 57:4 58:10 59:11 60:23 61:19 62:34 63:42</t>
+          <t>54:3 55:4 56:4 57:4 58:10 59:11 60:23 61:19 62:34 63:42 64:48 65:49 66:29 67:53 68:45 69:50 70:38 71:46 72:29 73:22 74:15 75:7 76:11 77:2 81:1 85:1</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>0:90 1:59 2:11 3:1 4:4 5:10 6:31 7:56 8:53 9:78 10:73 11:85 12:67 13:88 14:56 15:76 16:39 17:57 18:36 19:66 20:20 21:46 22:25 23:33 24:20 25:32 26:12 27:20 28:2 29:6 30:3 31:5 32:2</t>
+          <t>12:1 20:2 22:3 23:1 24:7 25:2 26:9 27:14 28:18 29:25 30:38 31:63 32:86 33:82 34:124 35:107 36:99 37:80 38:66 39:43 40:14 41:5 42:6 43:1 44:3 48:1</t>
         </is>
       </c>
     </row>
@@ -5050,67 +5038,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Orig Cubes</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Orig Literals</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Orig SSD</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ESOP Cubes</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ESOP Literals</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ESOP SSD</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ESOP SSD Saving (%)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Final Cubes</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Final Literals</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Final SSD</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>SSD Saving (%)</t>
         </is>
@@ -5577,16 +5565,16 @@
         <v>42.71</v>
       </c>
       <c r="J12" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K12" t="n">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="L12" t="n">
-        <v>0.06498619190316705</v>
+        <v>0.06093189964157706</v>
       </c>
       <c r="M12" t="n">
-        <v>86.98</v>
+        <v>87.79000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -5669,10 +5657,10 @@
         <v>188</v>
       </c>
       <c r="L14" t="n">
-        <v>0.05870511072147542</v>
+        <v>0.0583804143126177</v>
       </c>
       <c r="M14" t="n">
-        <v>88.23999999999999</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="15">
@@ -5712,10 +5700,10 @@
         <v>64</v>
       </c>
       <c r="L15" t="n">
-        <v>0.02070393374741201</v>
+        <v>0.01966873706004141</v>
       </c>
       <c r="M15" t="n">
-        <v>82.90000000000001</v>
+        <v>83.76000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -5755,10 +5743,10 @@
         <v>27</v>
       </c>
       <c r="L16" t="n">
-        <v>0.05</v>
+        <v>0.04722222222222222</v>
       </c>
       <c r="M16" t="n">
-        <v>89.95999999999999</v>
+        <v>90.52</v>
       </c>
     </row>
     <row r="17">
@@ -6056,10 +6044,10 @@
         <v>68</v>
       </c>
       <c r="L23" t="n">
-        <v>0.04532019704433497</v>
+        <v>0.04499178981937603</v>
       </c>
       <c r="M23" t="n">
-        <v>90.86</v>
+        <v>90.93000000000001</v>
       </c>
     </row>
     <row r="24">
@@ -6228,10 +6216,10 @@
         <v>124</v>
       </c>
       <c r="L27" t="n">
-        <v>0.05006938020351526</v>
+        <v>0.04949121184088807</v>
       </c>
       <c r="M27" t="n">
-        <v>89.95</v>
+        <v>90.06</v>
       </c>
     </row>
     <row r="28">
@@ -6311,13 +6299,13 @@
         <v>5</v>
       </c>
       <c r="K29" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="L29" t="n">
-        <v>0.06095238095238095</v>
+        <v>0.06571428571428571</v>
       </c>
       <c r="M29" t="n">
-        <v>87.8</v>
+        <v>86.84</v>
       </c>
     </row>
     <row r="30">
@@ -6354,13 +6342,13 @@
         <v>6</v>
       </c>
       <c r="K30" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L30" t="n">
-        <v>0.05751633986928104</v>
+        <v>0.05359477124183006</v>
       </c>
       <c r="M30" t="n">
-        <v>88.48999999999999</v>
+        <v>89.27</v>
       </c>
     </row>
     <row r="31">
@@ -6526,13 +6514,13 @@
         <v>41</v>
       </c>
       <c r="K34" t="n">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="L34" t="n">
-        <v>0.06245204336947456</v>
+        <v>0.06365304420350291</v>
       </c>
       <c r="M34" t="n">
-        <v>87.5</v>
+        <v>87.26000000000001</v>
       </c>
     </row>
     <row r="35">
@@ -6566,16 +6554,16 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>198</v>
+        <v>100</v>
       </c>
       <c r="K35" t="n">
-        <v>5511</v>
+        <v>10246</v>
       </c>
       <c r="L35" t="n">
-        <v>0.02651732515023654</v>
+        <v>0.0579489409141583</v>
       </c>
       <c r="M35" t="n">
-        <v>88.02</v>
+        <v>73.83</v>
       </c>
     </row>
     <row r="36">
@@ -6609,16 +6597,16 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>193</v>
+        <v>100</v>
       </c>
       <c r="K36" t="n">
-        <v>4430</v>
+        <v>10204</v>
       </c>
       <c r="L36" t="n">
-        <v>0.0239955752989307</v>
+        <v>0.05732976588628762</v>
       </c>
       <c r="M36" t="n">
-        <v>89.09999999999999</v>
+        <v>73.95</v>
       </c>
     </row>
     <row r="37">
@@ -6652,16 +6640,16 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>192</v>
+        <v>100</v>
       </c>
       <c r="K37" t="n">
-        <v>4399</v>
+        <v>10258</v>
       </c>
       <c r="L37" t="n">
-        <v>0.02109906899021246</v>
+        <v>0.05799152731326644</v>
       </c>
       <c r="M37" t="n">
-        <v>90.48999999999999</v>
+        <v>73.84999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -6695,16 +6683,16 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>197</v>
+        <v>100</v>
       </c>
       <c r="K38" t="n">
-        <v>5410</v>
+        <v>10183</v>
       </c>
       <c r="L38" t="n">
-        <v>0.02544774673538187</v>
+        <v>0.057120624303233</v>
       </c>
       <c r="M38" t="n">
-        <v>88.38</v>
+        <v>73.93000000000001</v>
       </c>
     </row>
     <row r="39">
@@ -6738,16 +6726,16 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>198</v>
+        <v>100</v>
       </c>
       <c r="K39" t="n">
-        <v>5394</v>
+        <v>10228</v>
       </c>
       <c r="L39" t="n">
-        <v>0.02557523152633007</v>
+        <v>0.05769453734671126</v>
       </c>
       <c r="M39" t="n">
-        <v>88.45999999999999</v>
+        <v>73.95999999999999</v>
       </c>
     </row>
     <row r="40">
@@ -6781,16 +6769,16 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>382</v>
+        <v>200</v>
       </c>
       <c r="K40" t="n">
-        <v>9990</v>
+        <v>20290</v>
       </c>
       <c r="L40" t="n">
-        <v>0.02211577217926984</v>
+        <v>0.05698920422927101</v>
       </c>
       <c r="M40" t="n">
-        <v>90.02</v>
+        <v>74.28</v>
       </c>
     </row>
     <row r="41">
@@ -6824,16 +6812,16 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>390</v>
+        <v>200</v>
       </c>
       <c r="K41" t="n">
-        <v>9991</v>
+        <v>20467</v>
       </c>
       <c r="L41" t="n">
-        <v>0.02460242890699185</v>
+        <v>0.05793656093489149</v>
       </c>
       <c r="M41" t="n">
-        <v>89.05</v>
+        <v>74.22</v>
       </c>
     </row>
     <row r="42">
@@ -6867,16 +6855,16 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>380</v>
+        <v>200</v>
       </c>
       <c r="K42" t="n">
-        <v>10160</v>
+        <v>20426</v>
       </c>
       <c r="L42" t="n">
-        <v>0.02246542553191489</v>
+        <v>0.05774451864218141</v>
       </c>
       <c r="M42" t="n">
-        <v>89.97</v>
+        <v>74.23</v>
       </c>
     </row>
     <row r="43">
@@ -6910,16 +6898,16 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>388</v>
+        <v>200</v>
       </c>
       <c r="K43" t="n">
-        <v>10065</v>
+        <v>20352</v>
       </c>
       <c r="L43" t="n">
-        <v>0.02378989402549532</v>
+        <v>0.05723539232053423</v>
       </c>
       <c r="M43" t="n">
-        <v>89.25</v>
+        <v>74.13</v>
       </c>
     </row>
     <row r="44">
@@ -6953,16 +6941,16 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>560</v>
+        <v>300</v>
       </c>
       <c r="K44" t="n">
-        <v>15502</v>
+        <v>30288</v>
       </c>
       <c r="L44" t="n">
-        <v>0.01998544122999548</v>
+        <v>0.05650997404523544</v>
       </c>
       <c r="M44" t="n">
-        <v>90.95999999999999</v>
+        <v>74.43000000000001</v>
       </c>
     </row>
     <row r="45">
@@ -6996,16 +6984,16 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>564</v>
+        <v>300</v>
       </c>
       <c r="K45" t="n">
-        <v>15414</v>
+        <v>30305</v>
       </c>
       <c r="L45" t="n">
-        <v>0.02109790932217617</v>
+        <v>0.05651294030404153</v>
       </c>
       <c r="M45" t="n">
-        <v>90.45</v>
+        <v>74.43000000000001</v>
       </c>
     </row>
     <row r="46">
@@ -7039,16 +7027,16 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>572</v>
+        <v>300</v>
       </c>
       <c r="K46" t="n">
-        <v>15642</v>
+        <v>30352</v>
       </c>
       <c r="L46" t="n">
-        <v>0.02249936190976654</v>
+        <v>0.05669227536769249</v>
       </c>
       <c r="M46" t="n">
-        <v>89.83</v>
+        <v>74.38</v>
       </c>
     </row>
     <row r="47">
@@ -7082,16 +7070,16 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>569</v>
+        <v>300</v>
       </c>
       <c r="K47" t="n">
-        <v>15676</v>
+        <v>30350</v>
       </c>
       <c r="L47" t="n">
-        <v>0.02173747078345536</v>
+        <v>0.05668540353479174</v>
       </c>
       <c r="M47" t="n">
-        <v>90.22</v>
+        <v>74.48999999999999</v>
       </c>
     </row>
     <row r="48">
@@ -7125,16 +7113,16 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>563</v>
+        <v>300</v>
       </c>
       <c r="K48" t="n">
-        <v>15616</v>
+        <v>30361</v>
       </c>
       <c r="L48" t="n">
-        <v>0.02066927990890936</v>
+        <v>0.05675998022494129</v>
       </c>
       <c r="M48" t="n">
-        <v>90.7</v>
+        <v>74.45999999999999</v>
       </c>
     </row>
     <row r="49">

</xml_diff>